<commit_message>
Accept newly scored actions
On behalf of V. Levy
</commit_message>
<xml_diff>
--- a/assessments/FinOps++/assessment.xlsx
+++ b/assessments/FinOps++/assessment.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="657" uniqueCount="275">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="929" uniqueCount="344">
   <si>
     <t>Sum of Weights</t>
   </si>
@@ -160,12 +160,39 @@
     <t>Prioritize Actions &amp; Publish Roadmap</t>
   </si>
   <si>
+    <t>Assess Skills &amp; Training Needs</t>
+  </si>
+  <si>
+    <t>Develop Role-Based Learning Content</t>
+  </si>
+  <si>
+    <t>Offer Certifications &amp; Informal Learning</t>
+  </si>
+  <si>
     <t>Leverage Vendor Training Resources</t>
   </si>
   <si>
+    <t>Track Training Impact &amp; Refresh Content</t>
+  </si>
+  <si>
     <t>Define Org Model &amp; Budget</t>
   </si>
   <si>
+    <t>Create Implementation Roadmap</t>
+  </si>
+  <si>
+    <t>Integrate Cost Data in Workflows</t>
+  </si>
+  <si>
+    <t>Publish FinOps KPIs</t>
+  </si>
+  <si>
+    <t>Drive Stakeholder Engagement</t>
+  </si>
+  <si>
+    <t>Automate Tasks &amp; Review Maturity</t>
+  </si>
+  <si>
     <t>Evaluate Build vs Buy Options</t>
   </si>
   <si>
@@ -193,9 +220,21 @@
     <t>Drive Adoption &amp; Resolve Conflicts</t>
   </si>
   <si>
+    <t>Map Invoices to Allocation Model</t>
+  </si>
+  <si>
+    <t>Reconcile Rates &amp; Track Completion</t>
+  </si>
+  <si>
     <t>Design Chargeback with Finance</t>
   </si>
   <si>
+    <t>Automate Chargeback Data Flows</t>
+  </si>
+  <si>
+    <t>Distribute Reports &amp; Track Accuracy</t>
+  </si>
+  <si>
     <t>Resolve Variances &amp; Increase Coverage</t>
   </si>
   <si>
@@ -211,15 +250,42 @@
     <t>Estimate Trade-Offs &amp; Document Cases</t>
   </si>
   <si>
+    <t>Create Workload Selection Criteria</t>
+  </si>
+  <si>
+    <t>Define Success Criteria &amp; Scope</t>
+  </si>
+  <si>
     <t>Enforce Tagging at Onboarding</t>
   </si>
   <si>
+    <t>Align Timelines with Budgets</t>
+  </si>
+  <si>
+    <t>Start with Lower Environments</t>
+  </si>
+  <si>
+    <t>Review Outcomes &amp; Adjust Patterns</t>
+  </si>
+  <si>
     <t>Inventory Licenses &amp; Map Resources</t>
   </si>
   <si>
+    <t>Document Licensing Models</t>
+  </si>
+  <si>
+    <t>Integrate Billing with Procurement</t>
+  </si>
+  <si>
     <t>Validate Utilization &amp; Remediate</t>
   </si>
   <si>
+    <t>Influence Workload Design Choices</t>
+  </si>
+  <si>
+    <t>Publish License Spend &amp; Utilization</t>
+  </si>
+  <si>
     <t>Document Commitment Strategy</t>
   </si>
   <si>
@@ -229,12 +295,24 @@
     <t>Leverage Spot &amp; Negotiated Discounts</t>
   </si>
   <si>
+    <t>Define Optimization Strategy</t>
+  </si>
+  <si>
     <t>Inventory &amp; Classify Workloads</t>
   </si>
   <si>
     <t>Collect Metrics &amp; Identify Candidates</t>
   </si>
   <si>
+    <t>Partner on Scheduling Actions</t>
+  </si>
+  <si>
+    <t>Gamify Adoption &amp; Celebrate Wins</t>
+  </si>
+  <si>
+    <t>Track KPIs &amp; Document Playbooks</t>
+  </si>
+  <si>
     <t>Define Metadata &amp; Hierarchy Strategy</t>
   </si>
   <si>
@@ -277,15 +355,27 @@
     <t>Define ingestion frequency; include mandatory metadata.</t>
   </si>
   <si>
+    <t>Gather Requirements &amp; Define KPIs</t>
+  </si>
+  <si>
     <t>Enrich Billing with Business Logic</t>
   </si>
   <si>
     <t>Build Dashboards for All Views</t>
   </si>
   <si>
+    <t>Publish Documentation &amp; Support</t>
+  </si>
+  <si>
     <t>Embed Reports in Workflows</t>
   </si>
   <si>
+    <t>Track Adoption &amp; Manage Changes</t>
+  </si>
+  <si>
+    <t>Iterate Based on Feedback</t>
+  </si>
+  <si>
     <t>Track Trends &amp; Compare Over Time</t>
   </si>
   <si>
@@ -295,6 +385,18 @@
     <t>Integrate Rolling Forecasts</t>
   </si>
   <si>
+    <t>Increase Shared Cost Coverage</t>
+  </si>
+  <si>
+    <t>Publish Budget vs Actual Reports</t>
+  </si>
+  <si>
+    <t>Automate Budget Threshold Alerts</t>
+  </si>
+  <si>
+    <t>Review &amp; Adapt Budget Strategy</t>
+  </si>
+  <si>
     <t>Collect Business Drivers Regularly</t>
   </si>
   <si>
@@ -364,12 +466,39 @@
     <t>116</t>
   </si>
   <si>
+    <t>097</t>
+  </si>
+  <si>
+    <t>098</t>
+  </si>
+  <si>
+    <t>099</t>
+  </si>
+  <si>
     <t>100</t>
   </si>
   <si>
+    <t>101</t>
+  </si>
+  <si>
     <t>091</t>
   </si>
   <si>
+    <t>092</t>
+  </si>
+  <si>
+    <t>093</t>
+  </si>
+  <si>
+    <t>094</t>
+  </si>
+  <si>
+    <t>095</t>
+  </si>
+  <si>
+    <t>096</t>
+  </si>
+  <si>
     <t>125</t>
   </si>
   <si>
@@ -397,9 +526,21 @@
     <t>134</t>
   </si>
   <si>
+    <t>107</t>
+  </si>
+  <si>
+    <t>108</t>
+  </si>
+  <si>
     <t>109</t>
   </si>
   <si>
+    <t>110</t>
+  </si>
+  <si>
+    <t>111</t>
+  </si>
+  <si>
     <t>112</t>
   </si>
   <si>
@@ -415,15 +556,42 @@
     <t>063</t>
   </si>
   <si>
+    <t>118</t>
+  </si>
+  <si>
+    <t>119</t>
+  </si>
+  <si>
     <t>120</t>
   </si>
   <si>
+    <t>121</t>
+  </si>
+  <si>
+    <t>122</t>
+  </si>
+  <si>
+    <t>123</t>
+  </si>
+  <si>
     <t>073</t>
   </si>
   <si>
+    <t>074</t>
+  </si>
+  <si>
+    <t>075</t>
+  </si>
+  <si>
     <t>076</t>
   </si>
   <si>
+    <t>077</t>
+  </si>
+  <si>
+    <t>078</t>
+  </si>
+  <si>
     <t>079</t>
   </si>
   <si>
@@ -433,12 +601,24 @@
     <t>084</t>
   </si>
   <si>
+    <t>067</t>
+  </si>
+  <si>
     <t>068</t>
   </si>
   <si>
     <t>069</t>
   </si>
   <si>
+    <t>070</t>
+  </si>
+  <si>
+    <t>071</t>
+  </si>
+  <si>
+    <t>072</t>
+  </si>
+  <si>
     <t>009</t>
   </si>
   <si>
@@ -481,15 +661,27 @@
     <t>135</t>
   </si>
   <si>
+    <t>016</t>
+  </si>
+  <si>
     <t>017</t>
   </si>
   <si>
     <t>018</t>
   </si>
   <si>
+    <t>019</t>
+  </si>
+  <si>
     <t>020</t>
   </si>
   <si>
+    <t>021</t>
+  </si>
+  <si>
+    <t>022</t>
+  </si>
+  <si>
     <t>053</t>
   </si>
   <si>
@@ -497,6 +689,18 @@
   </si>
   <si>
     <t>044</t>
+  </si>
+  <si>
+    <t>045</t>
+  </si>
+  <si>
+    <t>046</t>
+  </si>
+  <si>
+    <t>047</t>
+  </si>
+  <si>
+    <t>048</t>
   </si>
   <si>
     <t>038</t>
@@ -910,6 +1114,9 @@
   </si>
   <si>
     <t>[{'Score': 0, 'Condition': 'No items completed'}, {'Score': 3, 'Condition': 'item 1 completed'}, {'Score': 5, 'Condition': 'items 1-2 completed'}, {'Score': 8, 'Condition': 'items 1-3 completed'}, {'Score': 10, 'Condition': 'items 1-4 completed'}]</t>
+  </si>
+  <si>
+    <t>[{'Score': 0, 'Condition': 'Not done'}, {'Score': 10, 'Condition': 'Completed'}]</t>
   </si>
   <si>
     <t>[{'Score': 0, 'Condition': 'No items completed'}, {'Score': 5, 'Condition': '1 item completed'}, {'Score': 10, 'Condition': '2 items completed'}]</t>
@@ -1941,14 +2148,14 @@
     </row>
     <row r="2" spans="1:21">
       <c r="A2">
-        <f>SUM(Scoring!F2:F69)</f>
+        <f>SUM(Scoring!F2:F103)</f>
         <v>0</v>
       </c>
       <c r="B2">
         <v>10</v>
       </c>
       <c r="C2">
-        <f>SUM(Scoring!I2:I69)/A2</f>
+        <f>SUM(Scoring!I2:I103)/A2</f>
         <v>0</v>
       </c>
       <c r="D2">
@@ -1972,7 +2179,7 @@
         <v>1</v>
       </c>
       <c r="U5">
-        <f>SUMIF(Scoring!J2:J69,A5,Scoring!I2:I69)/SUMIF(Scoring!J2:J69,A5,Scoring!F2:F69)</f>
+        <f>SUMIF(Scoring!J2:J103,A5,Scoring!I2:I103)/SUMIF(Scoring!J2:J103,A5,Scoring!F2:F103)</f>
         <v>0</v>
       </c>
     </row>
@@ -1981,10 +2188,10 @@
         <v>7</v>
       </c>
       <c r="B6">
-        <v>18</v>
+        <v>31</v>
       </c>
       <c r="U6">
-        <f>SUMIF(Scoring!J2:J69,A6,Scoring!I2:I69)/SUMIF(Scoring!J2:J69,A6,Scoring!F2:F69)</f>
+        <f>SUMIF(Scoring!J2:J103,A6,Scoring!I2:I103)/SUMIF(Scoring!J2:J103,A6,Scoring!F2:F103)</f>
         <v>0</v>
       </c>
     </row>
@@ -1993,10 +2200,10 @@
         <v>8</v>
       </c>
       <c r="B7">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="U7">
-        <f>SUMIF(Scoring!J2:J69,A7,Scoring!I2:I69)/SUMIF(Scoring!J2:J69,A7,Scoring!F2:F69)</f>
+        <f>SUMIF(Scoring!J2:J103,A7,Scoring!I2:I103)/SUMIF(Scoring!J2:J103,A7,Scoring!F2:F103)</f>
         <v>0</v>
       </c>
     </row>
@@ -2005,10 +2212,10 @@
         <v>9</v>
       </c>
       <c r="B8">
-        <v>28</v>
+        <v>45</v>
       </c>
       <c r="U8">
-        <f>SUMIF(Scoring!J2:J69,A8,Scoring!I2:I69)/SUMIF(Scoring!J2:J69,A8,Scoring!F2:F69)</f>
+        <f>SUMIF(Scoring!J2:J103,A8,Scoring!I2:I103)/SUMIF(Scoring!J2:J103,A8,Scoring!F2:F103)</f>
         <v>0</v>
       </c>
     </row>
@@ -2034,7 +2241,7 @@
         <v>6</v>
       </c>
       <c r="U12">
-        <f>SUMIF(Scoring!K2:K69,A12,Scoring!I2:I69)/SUMIF(Scoring!K2:K69,A12,Scoring!F2:F69)</f>
+        <f>SUMIF(Scoring!K2:K103,A12,Scoring!I2:I103)/SUMIF(Scoring!K2:K103,A12,Scoring!F2:F103)</f>
         <v>0</v>
       </c>
     </row>
@@ -2046,7 +2253,7 @@
         <v>4</v>
       </c>
       <c r="U13">
-        <f>SUMIF(Scoring!K2:K69,A13,Scoring!I2:I69)/SUMIF(Scoring!K2:K69,A13,Scoring!F2:F69)</f>
+        <f>SUMIF(Scoring!K2:K103,A13,Scoring!I2:I103)/SUMIF(Scoring!K2:K103,A13,Scoring!F2:F103)</f>
         <v>0</v>
       </c>
     </row>
@@ -2055,10 +2262,10 @@
         <v>13</v>
       </c>
       <c r="B14">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="U14">
-        <f>SUMIF(Scoring!K2:K69,A14,Scoring!I2:I69)/SUMIF(Scoring!K2:K69,A14,Scoring!F2:F69)</f>
+        <f>SUMIF(Scoring!K2:K103,A14,Scoring!I2:I103)/SUMIF(Scoring!K2:K103,A14,Scoring!F2:F103)</f>
         <v>0</v>
       </c>
     </row>
@@ -2070,7 +2277,7 @@
         <v>3</v>
       </c>
       <c r="U15">
-        <f>SUMIF(Scoring!K2:K69,A15,Scoring!I2:I69)/SUMIF(Scoring!K2:K69,A15,Scoring!F2:F69)</f>
+        <f>SUMIF(Scoring!K2:K103,A15,Scoring!I2:I103)/SUMIF(Scoring!K2:K103,A15,Scoring!F2:F103)</f>
         <v>0</v>
       </c>
     </row>
@@ -2079,10 +2286,10 @@
         <v>15</v>
       </c>
       <c r="B16">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="U16">
-        <f>SUMIF(Scoring!K2:K69,A16,Scoring!I2:I69)/SUMIF(Scoring!K2:K69,A16,Scoring!F2:F69)</f>
+        <f>SUMIF(Scoring!K2:K103,A16,Scoring!I2:I103)/SUMIF(Scoring!K2:K103,A16,Scoring!F2:F103)</f>
         <v>0</v>
       </c>
     </row>
@@ -2094,7 +2301,7 @@
         <v>4</v>
       </c>
       <c r="U17">
-        <f>SUMIF(Scoring!K2:K69,A17,Scoring!I2:I69)/SUMIF(Scoring!K2:K69,A17,Scoring!F2:F69)</f>
+        <f>SUMIF(Scoring!K2:K103,A17,Scoring!I2:I103)/SUMIF(Scoring!K2:K103,A17,Scoring!F2:F103)</f>
         <v>0</v>
       </c>
     </row>
@@ -2106,7 +2313,7 @@
         <v>1</v>
       </c>
       <c r="U18">
-        <f>SUMIF(Scoring!K2:K69,A18,Scoring!I2:I69)/SUMIF(Scoring!K2:K69,A18,Scoring!F2:F69)</f>
+        <f>SUMIF(Scoring!K2:K103,A18,Scoring!I2:I103)/SUMIF(Scoring!K2:K103,A18,Scoring!F2:F103)</f>
         <v>0</v>
       </c>
     </row>
@@ -2118,7 +2325,7 @@
         <v>4</v>
       </c>
       <c r="U19">
-        <f>SUMIF(Scoring!K2:K69,A19,Scoring!I2:I69)/SUMIF(Scoring!K2:K69,A19,Scoring!F2:F69)</f>
+        <f>SUMIF(Scoring!K2:K103,A19,Scoring!I2:I103)/SUMIF(Scoring!K2:K103,A19,Scoring!F2:F103)</f>
         <v>0</v>
       </c>
     </row>
@@ -2127,10 +2334,10 @@
         <v>19</v>
       </c>
       <c r="B20">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="U20">
-        <f>SUMIF(Scoring!K2:K69,A20,Scoring!I2:I69)/SUMIF(Scoring!K2:K69,A20,Scoring!F2:F69)</f>
+        <f>SUMIF(Scoring!K2:K103,A20,Scoring!I2:I103)/SUMIF(Scoring!K2:K103,A20,Scoring!F2:F103)</f>
         <v>0</v>
       </c>
     </row>
@@ -2139,10 +2346,10 @@
         <v>20</v>
       </c>
       <c r="B21">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="U21">
-        <f>SUMIF(Scoring!K2:K69,A21,Scoring!I2:I69)/SUMIF(Scoring!K2:K69,A21,Scoring!F2:F69)</f>
+        <f>SUMIF(Scoring!K2:K103,A21,Scoring!I2:I103)/SUMIF(Scoring!K2:K103,A21,Scoring!F2:F103)</f>
         <v>0</v>
       </c>
     </row>
@@ -2154,7 +2361,7 @@
         <v>5</v>
       </c>
       <c r="U22">
-        <f>SUMIF(Scoring!K2:K69,A22,Scoring!I2:I69)/SUMIF(Scoring!K2:K69,A22,Scoring!F2:F69)</f>
+        <f>SUMIF(Scoring!K2:K103,A22,Scoring!I2:I103)/SUMIF(Scoring!K2:K103,A22,Scoring!F2:F103)</f>
         <v>0</v>
       </c>
     </row>
@@ -2166,7 +2373,7 @@
         <v>6</v>
       </c>
       <c r="U23">
-        <f>SUMIF(Scoring!K2:K69,A23,Scoring!I2:I69)/SUMIF(Scoring!K2:K69,A23,Scoring!F2:F69)</f>
+        <f>SUMIF(Scoring!K2:K103,A23,Scoring!I2:I103)/SUMIF(Scoring!K2:K103,A23,Scoring!F2:F103)</f>
         <v>0</v>
       </c>
     </row>
@@ -2175,10 +2382,10 @@
         <v>23</v>
       </c>
       <c r="B24">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="U24">
-        <f>SUMIF(Scoring!K2:K69,A24,Scoring!I2:I69)/SUMIF(Scoring!K2:K69,A24,Scoring!F2:F69)</f>
+        <f>SUMIF(Scoring!K2:K103,A24,Scoring!I2:I103)/SUMIF(Scoring!K2:K103,A24,Scoring!F2:F103)</f>
         <v>0</v>
       </c>
     </row>
@@ -2190,7 +2397,7 @@
         <v>1</v>
       </c>
       <c r="U25">
-        <f>SUMIF(Scoring!K2:K69,A25,Scoring!I2:I69)/SUMIF(Scoring!K2:K69,A25,Scoring!F2:F69)</f>
+        <f>SUMIF(Scoring!K2:K103,A25,Scoring!I2:I103)/SUMIF(Scoring!K2:K103,A25,Scoring!F2:F103)</f>
         <v>0</v>
       </c>
     </row>
@@ -2199,10 +2406,10 @@
         <v>25</v>
       </c>
       <c r="B26">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="U26">
-        <f>SUMIF(Scoring!K2:K69,A26,Scoring!I2:I69)/SUMIF(Scoring!K2:K69,A26,Scoring!F2:F69)</f>
+        <f>SUMIF(Scoring!K2:K103,A26,Scoring!I2:I103)/SUMIF(Scoring!K2:K103,A26,Scoring!F2:F103)</f>
         <v>0</v>
       </c>
     </row>
@@ -2214,7 +2421,7 @@
         <v>7</v>
       </c>
       <c r="U27">
-        <f>SUMIF(Scoring!K2:K69,A27,Scoring!I2:I69)/SUMIF(Scoring!K2:K69,A27,Scoring!F2:F69)</f>
+        <f>SUMIF(Scoring!K2:K103,A27,Scoring!I2:I103)/SUMIF(Scoring!K2:K103,A27,Scoring!F2:F103)</f>
         <v>0</v>
       </c>
     </row>
@@ -2226,7 +2433,7 @@
         <v>1</v>
       </c>
       <c r="U28">
-        <f>SUMIF(Scoring!K2:K69,A28,Scoring!I2:I69)/SUMIF(Scoring!K2:K69,A28,Scoring!F2:F69)</f>
+        <f>SUMIF(Scoring!K2:K103,A28,Scoring!I2:I103)/SUMIF(Scoring!K2:K103,A28,Scoring!F2:F103)</f>
         <v>0</v>
       </c>
     </row>
@@ -2238,7 +2445,7 @@
         <v>3</v>
       </c>
       <c r="U29">
-        <f>SUMIF(Scoring!K2:K69,A29,Scoring!I2:I69)/SUMIF(Scoring!K2:K69,A29,Scoring!F2:F69)</f>
+        <f>SUMIF(Scoring!K2:K103,A29,Scoring!I2:I103)/SUMIF(Scoring!K2:K103,A29,Scoring!F2:F103)</f>
         <v>0</v>
       </c>
     </row>
@@ -2247,10 +2454,10 @@
         <v>29</v>
       </c>
       <c r="B30">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="U30">
-        <f>SUMIF(Scoring!K2:K69,A30,Scoring!I2:I69)/SUMIF(Scoring!K2:K69,A30,Scoring!F2:F69)</f>
+        <f>SUMIF(Scoring!K2:K103,A30,Scoring!I2:I103)/SUMIF(Scoring!K2:K103,A30,Scoring!F2:F103)</f>
         <v>0</v>
       </c>
     </row>
@@ -2262,7 +2469,7 @@
         <v>6</v>
       </c>
       <c r="U31">
-        <f>SUMIF(Scoring!K2:K69,A31,Scoring!I2:I69)/SUMIF(Scoring!K2:K69,A31,Scoring!F2:F69)</f>
+        <f>SUMIF(Scoring!K2:K103,A31,Scoring!I2:I103)/SUMIF(Scoring!K2:K103,A31,Scoring!F2:F103)</f>
         <v>0</v>
       </c>
     </row>
@@ -2271,10 +2478,10 @@
         <v>31</v>
       </c>
       <c r="B32">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="U32">
-        <f>SUMIF(Scoring!K2:K69,A32,Scoring!I2:I69)/SUMIF(Scoring!K2:K69,A32,Scoring!F2:F69)</f>
+        <f>SUMIF(Scoring!K2:K103,A32,Scoring!I2:I103)/SUMIF(Scoring!K2:K103,A32,Scoring!F2:F103)</f>
         <v>0</v>
       </c>
     </row>
@@ -2297,7 +2504,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K69"/>
+  <dimension ref="A1:K103"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="25.42578125" bestFit="1" customWidth="1"/>
@@ -2359,19 +2566,19 @@
         <v>43</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>111</v>
+        <v>145</v>
       </c>
       <c r="E2" t="s">
-        <v>179</v>
+        <v>247</v>
       </c>
       <c r="F2">
         <v>1</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>183</v>
+        <v>251</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>258</v>
+        <v>327</v>
       </c>
       <c r="I2">
         <f>F2*VALUE(LEFT(H2, FIND(":", H2)-1))</f>
@@ -2391,19 +2598,19 @@
         <v>44</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>112</v>
+        <v>146</v>
       </c>
       <c r="E3" t="s">
-        <v>179</v>
+        <v>247</v>
       </c>
       <c r="F3">
         <v>1</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>184</v>
+        <v>252</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>259</v>
+        <v>328</v>
       </c>
       <c r="I3">
         <f>F3*VALUE(LEFT(H3, FIND(":", H3)-1))</f>
@@ -2423,19 +2630,19 @@
         <v>45</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>113</v>
+        <v>147</v>
       </c>
       <c r="E4" t="s">
-        <v>179</v>
+        <v>247</v>
       </c>
       <c r="F4">
         <v>1</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>185</v>
+        <v>253</v>
       </c>
       <c r="H4" s="1" t="s">
-        <v>259</v>
+        <v>328</v>
       </c>
       <c r="I4">
         <f>F4*VALUE(LEFT(H4, FIND(":", H4)-1))</f>
@@ -2455,19 +2662,19 @@
         <v>46</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>114</v>
+        <v>148</v>
       </c>
       <c r="E5" t="s">
-        <v>179</v>
+        <v>247</v>
       </c>
       <c r="F5">
         <v>1</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>186</v>
+        <v>254</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>259</v>
+        <v>328</v>
       </c>
       <c r="I5">
         <f>F5*VALUE(LEFT(H5, FIND(":", H5)-1))</f>
@@ -2489,19 +2696,16 @@
         <v>47</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>115</v>
+        <v>149</v>
       </c>
       <c r="E6" t="s">
-        <v>180</v>
+        <v>247</v>
       </c>
       <c r="F6">
         <v>1</v>
       </c>
-      <c r="G6" s="1" t="s">
-        <v>187</v>
-      </c>
       <c r="H6" s="1" t="s">
-        <v>259</v>
+        <v>329</v>
       </c>
       <c r="I6">
         <f>F6*VALUE(LEFT(H6, FIND(":", H6)-1))</f>
@@ -2516,23 +2720,21 @@
     </row>
     <row r="7" spans="1:11">
       <c r="A7" s="2"/>
-      <c r="B7" s="2" t="s">
-        <v>20</v>
-      </c>
+      <c r="B7" s="2"/>
       <c r="C7" s="2" t="s">
         <v>48</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>116</v>
+        <v>150</v>
       </c>
       <c r="E7" t="s">
-        <v>180</v>
+        <v>247</v>
       </c>
       <c r="F7">
         <v>1</v>
       </c>
       <c r="H7" s="1" t="s">
-        <v>260</v>
+        <v>329</v>
       </c>
       <c r="I7">
         <f>F7*VALUE(LEFT(H7, FIND(":", H7)-1))</f>
@@ -2542,31 +2744,26 @@
         <v>7</v>
       </c>
       <c r="K7" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="8" spans="1:11">
       <c r="A8" s="2"/>
-      <c r="B8" s="2" t="s">
-        <v>14</v>
-      </c>
+      <c r="B8" s="2"/>
       <c r="C8" s="2" t="s">
         <v>49</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>117</v>
+        <v>151</v>
       </c>
       <c r="E8" t="s">
-        <v>181</v>
+        <v>247</v>
       </c>
       <c r="F8">
         <v>1</v>
       </c>
-      <c r="G8" s="1" t="s">
-        <v>188</v>
-      </c>
       <c r="H8" s="1" t="s">
-        <v>261</v>
+        <v>329</v>
       </c>
       <c r="I8">
         <f>F8*VALUE(LEFT(H8, FIND(":", H8)-1))</f>
@@ -2576,7 +2773,7 @@
         <v>7</v>
       </c>
       <c r="K8" t="s">
-        <v>14</v>
+        <v>19</v>
       </c>
     </row>
     <row r="9" spans="1:11">
@@ -2586,19 +2783,19 @@
         <v>50</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>118</v>
+        <v>152</v>
       </c>
       <c r="E9" t="s">
-        <v>179</v>
+        <v>248</v>
       </c>
       <c r="F9">
         <v>1</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>189</v>
+        <v>255</v>
       </c>
       <c r="H9" s="1" t="s">
-        <v>262</v>
+        <v>328</v>
       </c>
       <c r="I9">
         <f>F9*VALUE(LEFT(H9, FIND(":", H9)-1))</f>
@@ -2608,7 +2805,7 @@
         <v>7</v>
       </c>
       <c r="K9" t="s">
-        <v>14</v>
+        <v>19</v>
       </c>
     </row>
     <row r="10" spans="1:11">
@@ -2618,19 +2815,16 @@
         <v>51</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>119</v>
+        <v>153</v>
       </c>
       <c r="E10" t="s">
-        <v>180</v>
+        <v>247</v>
       </c>
       <c r="F10">
         <v>1</v>
       </c>
-      <c r="G10" s="1" t="s">
-        <v>190</v>
-      </c>
       <c r="H10" s="1" t="s">
-        <v>259</v>
+        <v>329</v>
       </c>
       <c r="I10">
         <f>F10*VALUE(LEFT(H10, FIND(":", H10)-1))</f>
@@ -2640,31 +2834,28 @@
         <v>7</v>
       </c>
       <c r="K10" t="s">
-        <v>14</v>
+        <v>19</v>
       </c>
     </row>
     <row r="11" spans="1:11">
       <c r="A11" s="2"/>
       <c r="B11" s="2" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="C11" s="2" t="s">
         <v>52</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>120</v>
+        <v>154</v>
       </c>
       <c r="E11" t="s">
-        <v>179</v>
+        <v>248</v>
       </c>
       <c r="F11">
         <v>1</v>
       </c>
-      <c r="G11" s="1" t="s">
-        <v>191</v>
-      </c>
       <c r="H11" s="1" t="s">
-        <v>259</v>
+        <v>329</v>
       </c>
       <c r="I11">
         <f>F11*VALUE(LEFT(H11, FIND(":", H11)-1))</f>
@@ -2674,7 +2865,7 @@
         <v>7</v>
       </c>
       <c r="K11" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
     <row r="12" spans="1:11">
@@ -2684,19 +2875,16 @@
         <v>53</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>121</v>
+        <v>155</v>
       </c>
       <c r="E12" t="s">
-        <v>179</v>
+        <v>247</v>
       </c>
       <c r="F12">
         <v>1</v>
       </c>
-      <c r="G12" s="1" t="s">
-        <v>192</v>
-      </c>
       <c r="H12" s="1" t="s">
-        <v>259</v>
+        <v>329</v>
       </c>
       <c r="I12">
         <f>F12*VALUE(LEFT(H12, FIND(":", H12)-1))</f>
@@ -2706,7 +2894,7 @@
         <v>7</v>
       </c>
       <c r="K12" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
     <row r="13" spans="1:11">
@@ -2716,19 +2904,16 @@
         <v>54</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>122</v>
+        <v>156</v>
       </c>
       <c r="E13" t="s">
-        <v>179</v>
+        <v>247</v>
       </c>
       <c r="F13">
         <v>1</v>
       </c>
-      <c r="G13" s="1" t="s">
-        <v>193</v>
-      </c>
       <c r="H13" s="1" t="s">
-        <v>259</v>
+        <v>329</v>
       </c>
       <c r="I13">
         <f>F13*VALUE(LEFT(H13, FIND(":", H13)-1))</f>
@@ -2738,7 +2923,7 @@
         <v>7</v>
       </c>
       <c r="K13" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
     <row r="14" spans="1:11">
@@ -2748,19 +2933,16 @@
         <v>55</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>123</v>
+        <v>157</v>
       </c>
       <c r="E14" t="s">
-        <v>179</v>
+        <v>247</v>
       </c>
       <c r="F14">
         <v>1</v>
       </c>
-      <c r="G14" s="1" t="s">
-        <v>194</v>
-      </c>
       <c r="H14" s="1" t="s">
-        <v>259</v>
+        <v>329</v>
       </c>
       <c r="I14">
         <f>F14*VALUE(LEFT(H14, FIND(":", H14)-1))</f>
@@ -2770,7 +2952,7 @@
         <v>7</v>
       </c>
       <c r="K14" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
     <row r="15" spans="1:11">
@@ -2780,19 +2962,16 @@
         <v>56</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>124</v>
+        <v>158</v>
       </c>
       <c r="E15" t="s">
-        <v>179</v>
+        <v>247</v>
       </c>
       <c r="F15">
         <v>1</v>
       </c>
-      <c r="G15" s="1" t="s">
-        <v>195</v>
-      </c>
       <c r="H15" s="1" t="s">
-        <v>259</v>
+        <v>329</v>
       </c>
       <c r="I15">
         <f>F15*VALUE(LEFT(H15, FIND(":", H15)-1))</f>
@@ -2802,7 +2981,7 @@
         <v>7</v>
       </c>
       <c r="K15" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
     <row r="16" spans="1:11">
@@ -2812,19 +2991,16 @@
         <v>57</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>125</v>
+        <v>159</v>
       </c>
       <c r="E16" t="s">
-        <v>179</v>
+        <v>247</v>
       </c>
       <c r="F16">
         <v>1</v>
       </c>
-      <c r="G16" s="1" t="s">
-        <v>196</v>
-      </c>
       <c r="H16" s="1" t="s">
-        <v>259</v>
+        <v>329</v>
       </c>
       <c r="I16">
         <f>F16*VALUE(LEFT(H16, FIND(":", H16)-1))</f>
@@ -2834,28 +3010,31 @@
         <v>7</v>
       </c>
       <c r="K16" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
     <row r="17" spans="1:11">
       <c r="A17" s="2"/>
       <c r="B17" s="2" t="s">
-        <v>23</v>
+        <v>14</v>
       </c>
       <c r="C17" s="2" t="s">
         <v>58</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>126</v>
+        <v>160</v>
       </c>
       <c r="E17" t="s">
-        <v>180</v>
+        <v>249</v>
       </c>
       <c r="F17">
         <v>1</v>
       </c>
+      <c r="G17" s="1" t="s">
+        <v>256</v>
+      </c>
       <c r="H17" s="1" t="s">
-        <v>260</v>
+        <v>330</v>
       </c>
       <c r="I17">
         <f>F17*VALUE(LEFT(H17, FIND(":", H17)-1))</f>
@@ -2865,7 +3044,7 @@
         <v>7</v>
       </c>
       <c r="K17" t="s">
-        <v>23</v>
+        <v>14</v>
       </c>
     </row>
     <row r="18" spans="1:11">
@@ -2875,16 +3054,19 @@
         <v>59</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>127</v>
+        <v>161</v>
       </c>
       <c r="E18" t="s">
-        <v>180</v>
+        <v>247</v>
       </c>
       <c r="F18">
         <v>1</v>
       </c>
+      <c r="G18" s="1" t="s">
+        <v>257</v>
+      </c>
       <c r="H18" s="1" t="s">
-        <v>260</v>
+        <v>331</v>
       </c>
       <c r="I18">
         <f>F18*VALUE(LEFT(H18, FIND(":", H18)-1))</f>
@@ -2894,28 +3076,29 @@
         <v>7</v>
       </c>
       <c r="K18" t="s">
-        <v>23</v>
+        <v>14</v>
       </c>
     </row>
     <row r="19" spans="1:11">
       <c r="A19" s="2"/>
-      <c r="B19" s="2" t="s">
-        <v>17</v>
-      </c>
+      <c r="B19" s="2"/>
       <c r="C19" s="2" t="s">
         <v>60</v>
       </c>
       <c r="D19" s="3" t="s">
-        <v>128</v>
+        <v>162</v>
       </c>
       <c r="E19" t="s">
-        <v>179</v>
+        <v>248</v>
       </c>
       <c r="F19">
         <v>1</v>
       </c>
+      <c r="G19" s="1" t="s">
+        <v>258</v>
+      </c>
       <c r="H19" s="1" t="s">
-        <v>263</v>
+        <v>328</v>
       </c>
       <c r="I19">
         <f>F19*VALUE(LEFT(H19, FIND(":", H19)-1))</f>
@@ -2925,40 +3108,41 @@
         <v>7</v>
       </c>
       <c r="K19" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
     </row>
     <row r="20" spans="1:11">
-      <c r="A20" s="2" t="s">
-        <v>9</v>
-      </c>
+      <c r="A20" s="2"/>
       <c r="B20" s="2" t="s">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="C20" s="2" t="s">
         <v>61</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>129</v>
+        <v>163</v>
       </c>
       <c r="E20" t="s">
-        <v>180</v>
+        <v>247</v>
       </c>
       <c r="F20">
         <v>1</v>
       </c>
+      <c r="G20" s="1" t="s">
+        <v>259</v>
+      </c>
       <c r="H20" s="1" t="s">
-        <v>264</v>
+        <v>328</v>
       </c>
       <c r="I20">
         <f>F20*VALUE(LEFT(H20, FIND(":", H20)-1))</f>
         <v>0</v>
       </c>
       <c r="J20" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="K20" t="s">
-        <v>13</v>
+        <v>22</v>
       </c>
     </row>
     <row r="21" spans="1:11">
@@ -2968,29 +3152,29 @@
         <v>62</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>130</v>
+        <v>164</v>
       </c>
       <c r="E21" t="s">
-        <v>180</v>
+        <v>247</v>
       </c>
       <c r="F21">
         <v>1</v>
       </c>
       <c r="G21" s="1" t="s">
-        <v>197</v>
+        <v>260</v>
       </c>
       <c r="H21" s="1" t="s">
-        <v>259</v>
+        <v>328</v>
       </c>
       <c r="I21">
         <f>F21*VALUE(LEFT(H21, FIND(":", H21)-1))</f>
         <v>0</v>
       </c>
       <c r="J21" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="K21" t="s">
-        <v>13</v>
+        <v>22</v>
       </c>
     </row>
     <row r="22" spans="1:11">
@@ -3000,26 +3184,29 @@
         <v>63</v>
       </c>
       <c r="D22" s="3" t="s">
-        <v>131</v>
+        <v>165</v>
       </c>
       <c r="E22" t="s">
-        <v>180</v>
+        <v>247</v>
       </c>
       <c r="F22">
         <v>1</v>
       </c>
+      <c r="G22" s="1" t="s">
+        <v>261</v>
+      </c>
       <c r="H22" s="1" t="s">
-        <v>265</v>
+        <v>328</v>
       </c>
       <c r="I22">
         <f>F22*VALUE(LEFT(H22, FIND(":", H22)-1))</f>
         <v>0</v>
       </c>
       <c r="J22" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="K22" t="s">
-        <v>13</v>
+        <v>22</v>
       </c>
     </row>
     <row r="23" spans="1:11">
@@ -3029,60 +3216,61 @@
         <v>64</v>
       </c>
       <c r="D23" s="3" t="s">
-        <v>132</v>
+        <v>166</v>
       </c>
       <c r="E23" t="s">
-        <v>180</v>
+        <v>247</v>
       </c>
       <c r="F23">
         <v>1</v>
       </c>
       <c r="G23" s="1" t="s">
-        <v>198</v>
+        <v>262</v>
       </c>
       <c r="H23" s="1" t="s">
-        <v>259</v>
+        <v>328</v>
       </c>
       <c r="I23">
         <f>F23*VALUE(LEFT(H23, FIND(":", H23)-1))</f>
         <v>0</v>
       </c>
       <c r="J23" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="K23" t="s">
-        <v>13</v>
+        <v>22</v>
       </c>
     </row>
     <row r="24" spans="1:11">
       <c r="A24" s="2"/>
-      <c r="B24" s="2" t="s">
-        <v>25</v>
-      </c>
+      <c r="B24" s="2"/>
       <c r="C24" s="2" t="s">
         <v>65</v>
       </c>
       <c r="D24" s="3" t="s">
-        <v>133</v>
+        <v>167</v>
       </c>
       <c r="E24" t="s">
-        <v>180</v>
+        <v>247</v>
       </c>
       <c r="F24">
         <v>1</v>
       </c>
+      <c r="G24" s="1" t="s">
+        <v>263</v>
+      </c>
       <c r="H24" s="1" t="s">
-        <v>266</v>
+        <v>328</v>
       </c>
       <c r="I24">
         <f>F24*VALUE(LEFT(H24, FIND(":", H24)-1))</f>
         <v>0</v>
       </c>
       <c r="J24" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="K24" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
     </row>
     <row r="25" spans="1:11">
@@ -3092,57 +3280,60 @@
         <v>66</v>
       </c>
       <c r="D25" s="3" t="s">
-        <v>134</v>
+        <v>168</v>
       </c>
       <c r="E25" t="s">
-        <v>180</v>
+        <v>247</v>
       </c>
       <c r="F25">
         <v>1</v>
       </c>
+      <c r="G25" s="1" t="s">
+        <v>264</v>
+      </c>
       <c r="H25" s="1" t="s">
-        <v>260</v>
+        <v>328</v>
       </c>
       <c r="I25">
         <f>F25*VALUE(LEFT(H25, FIND(":", H25)-1))</f>
         <v>0</v>
       </c>
       <c r="J25" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="K25" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
     </row>
     <row r="26" spans="1:11">
       <c r="A26" s="2"/>
       <c r="B26" s="2" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="C26" s="2" t="s">
         <v>67</v>
       </c>
       <c r="D26" s="3" t="s">
-        <v>135</v>
+        <v>169</v>
       </c>
       <c r="E26" t="s">
-        <v>180</v>
+        <v>247</v>
       </c>
       <c r="F26">
         <v>1</v>
       </c>
       <c r="H26" s="1" t="s">
-        <v>260</v>
+        <v>329</v>
       </c>
       <c r="I26">
         <f>F26*VALUE(LEFT(H26, FIND(":", H26)-1))</f>
         <v>0</v>
       </c>
       <c r="J26" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="K26" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
     </row>
     <row r="27" spans="1:11">
@@ -3152,26 +3343,26 @@
         <v>68</v>
       </c>
       <c r="D27" s="3" t="s">
-        <v>136</v>
+        <v>170</v>
       </c>
       <c r="E27" t="s">
-        <v>180</v>
+        <v>247</v>
       </c>
       <c r="F27">
         <v>1</v>
       </c>
       <c r="H27" s="1" t="s">
-        <v>260</v>
+        <v>329</v>
       </c>
       <c r="I27">
         <f>F27*VALUE(LEFT(H27, FIND(":", H27)-1))</f>
         <v>0</v>
       </c>
       <c r="J27" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="K27" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
     </row>
     <row r="28" spans="1:11">
@@ -3181,60 +3372,55 @@
         <v>69</v>
       </c>
       <c r="D28" s="3" t="s">
-        <v>137</v>
+        <v>171</v>
       </c>
       <c r="E28" t="s">
-        <v>180</v>
+        <v>248</v>
       </c>
       <c r="F28">
         <v>1</v>
       </c>
-      <c r="G28" s="1" t="s">
-        <v>199</v>
-      </c>
       <c r="H28" s="1" t="s">
-        <v>259</v>
+        <v>329</v>
       </c>
       <c r="I28">
         <f>F28*VALUE(LEFT(H28, FIND(":", H28)-1))</f>
         <v>0</v>
       </c>
       <c r="J28" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="K28" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
     </row>
     <row r="29" spans="1:11">
       <c r="A29" s="2"/>
-      <c r="B29" s="2" t="s">
-        <v>31</v>
-      </c>
+      <c r="B29" s="2"/>
       <c r="C29" s="2" t="s">
         <v>70</v>
       </c>
       <c r="D29" s="3" t="s">
-        <v>138</v>
+        <v>172</v>
       </c>
       <c r="E29" t="s">
-        <v>180</v>
+        <v>247</v>
       </c>
       <c r="F29">
         <v>1</v>
       </c>
       <c r="H29" s="1" t="s">
-        <v>267</v>
+        <v>329</v>
       </c>
       <c r="I29">
         <f>F29*VALUE(LEFT(H29, FIND(":", H29)-1))</f>
         <v>0</v>
       </c>
       <c r="J29" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="K29" t="s">
-        <v>31</v>
+        <v>23</v>
       </c>
     </row>
     <row r="30" spans="1:11">
@@ -3244,114 +3430,109 @@
         <v>71</v>
       </c>
       <c r="D30" s="3" t="s">
-        <v>139</v>
+        <v>173</v>
       </c>
       <c r="E30" t="s">
-        <v>180</v>
+        <v>247</v>
       </c>
       <c r="F30">
         <v>1</v>
       </c>
       <c r="H30" s="1" t="s">
-        <v>266</v>
+        <v>329</v>
       </c>
       <c r="I30">
         <f>F30*VALUE(LEFT(H30, FIND(":", H30)-1))</f>
         <v>0</v>
       </c>
       <c r="J30" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="K30" t="s">
-        <v>31</v>
+        <v>23</v>
       </c>
     </row>
     <row r="31" spans="1:11">
       <c r="A31" s="2"/>
-      <c r="B31" s="2" t="s">
-        <v>11</v>
-      </c>
+      <c r="B31" s="2"/>
       <c r="C31" s="2" t="s">
         <v>72</v>
       </c>
       <c r="D31" s="3" t="s">
-        <v>140</v>
+        <v>174</v>
       </c>
       <c r="E31" t="s">
-        <v>180</v>
+        <v>248</v>
       </c>
       <c r="F31">
         <v>1</v>
       </c>
-      <c r="G31" s="1" t="s">
-        <v>200</v>
-      </c>
       <c r="H31" s="1" t="s">
-        <v>259</v>
+        <v>329</v>
       </c>
       <c r="I31">
         <f>F31*VALUE(LEFT(H31, FIND(":", H31)-1))</f>
         <v>0</v>
       </c>
       <c r="J31" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="K31" t="s">
-        <v>11</v>
+        <v>23</v>
       </c>
     </row>
     <row r="32" spans="1:11">
       <c r="A32" s="2"/>
-      <c r="B32" s="2"/>
+      <c r="B32" s="2" t="s">
+        <v>17</v>
+      </c>
       <c r="C32" s="2" t="s">
         <v>73</v>
       </c>
       <c r="D32" s="3" t="s">
-        <v>141</v>
+        <v>175</v>
       </c>
       <c r="E32" t="s">
-        <v>180</v>
+        <v>247</v>
       </c>
       <c r="F32">
         <v>1</v>
       </c>
-      <c r="G32" s="1" t="s">
-        <v>201</v>
-      </c>
       <c r="H32" s="1" t="s">
-        <v>266</v>
+        <v>332</v>
       </c>
       <c r="I32">
         <f>F32*VALUE(LEFT(H32, FIND(":", H32)-1))</f>
         <v>0</v>
       </c>
       <c r="J32" t="s">
+        <v>7</v>
+      </c>
+      <c r="K32" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="33" spans="1:11">
+      <c r="A33" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="K32" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="33" spans="1:11">
-      <c r="A33" s="2"/>
-      <c r="B33" s="2"/>
+      <c r="B33" s="2" t="s">
+        <v>13</v>
+      </c>
       <c r="C33" s="2" t="s">
         <v>74</v>
       </c>
       <c r="D33" s="3" t="s">
-        <v>142</v>
+        <v>176</v>
       </c>
       <c r="E33" t="s">
-        <v>180</v>
+        <v>248</v>
       </c>
       <c r="F33">
         <v>1</v>
       </c>
-      <c r="G33" s="1" t="s">
-        <v>202</v>
-      </c>
       <c r="H33" s="1" t="s">
-        <v>259</v>
+        <v>333</v>
       </c>
       <c r="I33">
         <f>F33*VALUE(LEFT(H33, FIND(":", H33)-1))</f>
@@ -3361,7 +3542,7 @@
         <v>9</v>
       </c>
       <c r="K33" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
     </row>
     <row r="34" spans="1:11">
@@ -3371,19 +3552,19 @@
         <v>75</v>
       </c>
       <c r="D34" s="3" t="s">
-        <v>143</v>
+        <v>177</v>
       </c>
       <c r="E34" t="s">
-        <v>180</v>
+        <v>248</v>
       </c>
       <c r="F34">
         <v>1</v>
       </c>
       <c r="G34" s="1" t="s">
-        <v>203</v>
+        <v>265</v>
       </c>
       <c r="H34" s="1" t="s">
-        <v>266</v>
+        <v>328</v>
       </c>
       <c r="I34">
         <f>F34*VALUE(LEFT(H34, FIND(":", H34)-1))</f>
@@ -3393,7 +3574,7 @@
         <v>9</v>
       </c>
       <c r="K34" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
     </row>
     <row r="35" spans="1:11">
@@ -3403,19 +3584,16 @@
         <v>76</v>
       </c>
       <c r="D35" s="3" t="s">
-        <v>144</v>
+        <v>178</v>
       </c>
       <c r="E35" t="s">
-        <v>180</v>
+        <v>248</v>
       </c>
       <c r="F35">
         <v>1</v>
       </c>
-      <c r="G35" s="1" t="s">
-        <v>204</v>
-      </c>
       <c r="H35" s="1" t="s">
-        <v>266</v>
+        <v>334</v>
       </c>
       <c r="I35">
         <f>F35*VALUE(LEFT(H35, FIND(":", H35)-1))</f>
@@ -3425,7 +3603,7 @@
         <v>9</v>
       </c>
       <c r="K35" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
     </row>
     <row r="36" spans="1:11">
@@ -3435,19 +3613,16 @@
         <v>77</v>
       </c>
       <c r="D36" s="3" t="s">
-        <v>145</v>
+        <v>179</v>
       </c>
       <c r="E36" t="s">
-        <v>180</v>
+        <v>247</v>
       </c>
       <c r="F36">
         <v>1</v>
       </c>
-      <c r="G36" s="1" t="s">
-        <v>205</v>
-      </c>
       <c r="H36" s="1" t="s">
-        <v>259</v>
+        <v>329</v>
       </c>
       <c r="I36">
         <f>F36*VALUE(LEFT(H36, FIND(":", H36)-1))</f>
@@ -3457,31 +3632,26 @@
         <v>9</v>
       </c>
       <c r="K36" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
     </row>
     <row r="37" spans="1:11">
       <c r="A37" s="2"/>
-      <c r="B37" s="2" t="s">
-        <v>12</v>
-      </c>
+      <c r="B37" s="2"/>
       <c r="C37" s="2" t="s">
         <v>78</v>
       </c>
       <c r="D37" s="3" t="s">
-        <v>146</v>
+        <v>180</v>
       </c>
       <c r="E37" t="s">
-        <v>180</v>
+        <v>247</v>
       </c>
       <c r="F37">
         <v>1</v>
       </c>
-      <c r="G37" s="1" t="s">
-        <v>206</v>
-      </c>
       <c r="H37" s="1" t="s">
-        <v>259</v>
+        <v>329</v>
       </c>
       <c r="I37">
         <f>F37*VALUE(LEFT(H37, FIND(":", H37)-1))</f>
@@ -3491,7 +3661,7 @@
         <v>9</v>
       </c>
       <c r="K37" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="38" spans="1:11">
@@ -3501,19 +3671,19 @@
         <v>79</v>
       </c>
       <c r="D38" s="3" t="s">
-        <v>147</v>
+        <v>181</v>
       </c>
       <c r="E38" t="s">
-        <v>180</v>
+        <v>248</v>
       </c>
       <c r="F38">
         <v>1</v>
       </c>
       <c r="G38" s="1" t="s">
-        <v>207</v>
+        <v>266</v>
       </c>
       <c r="H38" s="1" t="s">
-        <v>259</v>
+        <v>328</v>
       </c>
       <c r="I38">
         <f>F38*VALUE(LEFT(H38, FIND(":", H38)-1))</f>
@@ -3523,7 +3693,7 @@
         <v>9</v>
       </c>
       <c r="K38" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="39" spans="1:11">
@@ -3533,16 +3703,16 @@
         <v>80</v>
       </c>
       <c r="D39" s="3" t="s">
-        <v>148</v>
+        <v>182</v>
       </c>
       <c r="E39" t="s">
-        <v>180</v>
+        <v>247</v>
       </c>
       <c r="F39">
         <v>1</v>
       </c>
       <c r="H39" s="1" t="s">
-        <v>268</v>
+        <v>329</v>
       </c>
       <c r="I39">
         <f>F39*VALUE(LEFT(H39, FIND(":", H39)-1))</f>
@@ -3552,7 +3722,7 @@
         <v>9</v>
       </c>
       <c r="K39" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="40" spans="1:11">
@@ -3562,19 +3732,16 @@
         <v>81</v>
       </c>
       <c r="D40" s="3" t="s">
-        <v>149</v>
+        <v>183</v>
       </c>
       <c r="E40" t="s">
-        <v>180</v>
+        <v>247</v>
       </c>
       <c r="F40">
         <v>1</v>
       </c>
-      <c r="G40" s="1" t="s">
-        <v>208</v>
-      </c>
       <c r="H40" s="1" t="s">
-        <v>259</v>
+        <v>329</v>
       </c>
       <c r="I40">
         <f>F40*VALUE(LEFT(H40, FIND(":", H40)-1))</f>
@@ -3584,28 +3751,26 @@
         <v>9</v>
       </c>
       <c r="K40" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="41" spans="1:11">
       <c r="A41" s="2"/>
-      <c r="B41" s="2" t="s">
-        <v>16</v>
-      </c>
+      <c r="B41" s="2"/>
       <c r="C41" s="2" t="s">
         <v>82</v>
       </c>
       <c r="D41" s="3" t="s">
-        <v>150</v>
+        <v>184</v>
       </c>
       <c r="E41" t="s">
-        <v>180</v>
+        <v>247</v>
       </c>
       <c r="F41">
         <v>1</v>
       </c>
       <c r="H41" s="1" t="s">
-        <v>269</v>
+        <v>329</v>
       </c>
       <c r="I41">
         <f>F41*VALUE(LEFT(H41, FIND(":", H41)-1))</f>
@@ -3615,29 +3780,28 @@
         <v>9</v>
       </c>
       <c r="K41" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
     </row>
     <row r="42" spans="1:11">
       <c r="A42" s="2"/>
-      <c r="B42" s="2"/>
+      <c r="B42" s="2" t="s">
+        <v>25</v>
+      </c>
       <c r="C42" s="2" t="s">
         <v>83</v>
       </c>
       <c r="D42" s="3" t="s">
-        <v>151</v>
+        <v>185</v>
       </c>
       <c r="E42" t="s">
-        <v>180</v>
+        <v>248</v>
       </c>
       <c r="F42">
         <v>1</v>
       </c>
-      <c r="G42" s="1" t="s">
-        <v>209</v>
-      </c>
       <c r="H42" s="1" t="s">
-        <v>259</v>
+        <v>335</v>
       </c>
       <c r="I42">
         <f>F42*VALUE(LEFT(H42, FIND(":", H42)-1))</f>
@@ -3647,7 +3811,7 @@
         <v>9</v>
       </c>
       <c r="K42" t="s">
-        <v>16</v>
+        <v>25</v>
       </c>
     </row>
     <row r="43" spans="1:11">
@@ -3657,19 +3821,16 @@
         <v>84</v>
       </c>
       <c r="D43" s="3" t="s">
-        <v>152</v>
+        <v>186</v>
       </c>
       <c r="E43" t="s">
-        <v>180</v>
+        <v>247</v>
       </c>
       <c r="F43">
         <v>1</v>
       </c>
-      <c r="G43" s="1" t="s">
-        <v>210</v>
-      </c>
       <c r="H43" s="1" t="s">
-        <v>259</v>
+        <v>329</v>
       </c>
       <c r="I43">
         <f>F43*VALUE(LEFT(H43, FIND(":", H43)-1))</f>
@@ -3679,7 +3840,7 @@
         <v>9</v>
       </c>
       <c r="K43" t="s">
-        <v>16</v>
+        <v>25</v>
       </c>
     </row>
     <row r="44" spans="1:11">
@@ -3689,16 +3850,16 @@
         <v>85</v>
       </c>
       <c r="D44" s="3" t="s">
-        <v>153</v>
+        <v>187</v>
       </c>
       <c r="E44" t="s">
-        <v>182</v>
+        <v>247</v>
       </c>
       <c r="F44">
         <v>1</v>
       </c>
       <c r="H44" s="1" t="s">
-        <v>269</v>
+        <v>329</v>
       </c>
       <c r="I44">
         <f>F44*VALUE(LEFT(H44, FIND(":", H44)-1))</f>
@@ -3708,31 +3869,26 @@
         <v>9</v>
       </c>
       <c r="K44" t="s">
-        <v>16</v>
+        <v>25</v>
       </c>
     </row>
     <row r="45" spans="1:11">
       <c r="A45" s="2"/>
-      <c r="B45" s="2" t="s">
-        <v>29</v>
-      </c>
+      <c r="B45" s="2"/>
       <c r="C45" s="2" t="s">
         <v>86</v>
       </c>
       <c r="D45" s="3" t="s">
-        <v>154</v>
+        <v>188</v>
       </c>
       <c r="E45" t="s">
-        <v>180</v>
+        <v>248</v>
       </c>
       <c r="F45">
         <v>1</v>
       </c>
-      <c r="G45" s="1" t="s">
-        <v>211</v>
-      </c>
       <c r="H45" s="1" t="s">
-        <v>259</v>
+        <v>329</v>
       </c>
       <c r="I45">
         <f>F45*VALUE(LEFT(H45, FIND(":", H45)-1))</f>
@@ -3742,7 +3898,7 @@
         <v>9</v>
       </c>
       <c r="K45" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
     </row>
     <row r="46" spans="1:11">
@@ -3752,19 +3908,16 @@
         <v>87</v>
       </c>
       <c r="D46" s="3" t="s">
-        <v>155</v>
+        <v>189</v>
       </c>
       <c r="E46" t="s">
-        <v>180</v>
+        <v>247</v>
       </c>
       <c r="F46">
         <v>1</v>
       </c>
-      <c r="G46" s="1" t="s">
-        <v>212</v>
-      </c>
       <c r="H46" s="1" t="s">
-        <v>259</v>
+        <v>329</v>
       </c>
       <c r="I46">
         <f>F46*VALUE(LEFT(H46, FIND(":", H46)-1))</f>
@@ -3774,7 +3927,7 @@
         <v>9</v>
       </c>
       <c r="K46" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
     </row>
     <row r="47" spans="1:11">
@@ -3784,16 +3937,16 @@
         <v>88</v>
       </c>
       <c r="D47" s="3" t="s">
-        <v>156</v>
+        <v>190</v>
       </c>
       <c r="E47" t="s">
-        <v>180</v>
+        <v>247</v>
       </c>
       <c r="F47">
         <v>1</v>
       </c>
       <c r="H47" s="1" t="s">
-        <v>270</v>
+        <v>329</v>
       </c>
       <c r="I47">
         <f>F47*VALUE(LEFT(H47, FIND(":", H47)-1))</f>
@@ -3803,71 +3956,67 @@
         <v>9</v>
       </c>
       <c r="K47" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
     </row>
     <row r="48" spans="1:11">
-      <c r="A48" s="2" t="s">
-        <v>8</v>
-      </c>
+      <c r="A48" s="2"/>
       <c r="B48" s="2" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="C48" s="2" t="s">
         <v>89</v>
       </c>
       <c r="D48" s="3" t="s">
-        <v>157</v>
+        <v>191</v>
       </c>
       <c r="E48" t="s">
-        <v>180</v>
+        <v>248</v>
       </c>
       <c r="F48">
         <v>1</v>
       </c>
       <c r="H48" s="1" t="s">
-        <v>271</v>
+        <v>329</v>
       </c>
       <c r="I48">
         <f>F48*VALUE(LEFT(H48, FIND(":", H48)-1))</f>
         <v>0</v>
       </c>
       <c r="J48" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="K48" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
     </row>
     <row r="49" spans="1:11">
       <c r="A49" s="2"/>
-      <c r="B49" s="2" t="s">
-        <v>15</v>
-      </c>
+      <c r="B49" s="2"/>
       <c r="C49" s="2" t="s">
         <v>90</v>
       </c>
       <c r="D49" s="3" t="s">
-        <v>158</v>
+        <v>192</v>
       </c>
       <c r="E49" t="s">
-        <v>180</v>
+        <v>248</v>
       </c>
       <c r="F49">
         <v>1</v>
       </c>
       <c r="H49" s="1" t="s">
-        <v>264</v>
+        <v>329</v>
       </c>
       <c r="I49">
         <f>F49*VALUE(LEFT(H49, FIND(":", H49)-1))</f>
         <v>0</v>
       </c>
       <c r="J49" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="K49" t="s">
-        <v>15</v>
+        <v>28</v>
       </c>
     </row>
     <row r="50" spans="1:11">
@@ -3877,60 +4026,60 @@
         <v>91</v>
       </c>
       <c r="D50" s="3" t="s">
-        <v>159</v>
+        <v>193</v>
       </c>
       <c r="E50" t="s">
-        <v>180</v>
+        <v>248</v>
       </c>
       <c r="F50">
         <v>1</v>
       </c>
+      <c r="G50" s="1" t="s">
+        <v>267</v>
+      </c>
       <c r="H50" s="1" t="s">
-        <v>264</v>
+        <v>328</v>
       </c>
       <c r="I50">
         <f>F50*VALUE(LEFT(H50, FIND(":", H50)-1))</f>
         <v>0</v>
       </c>
       <c r="J50" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="K50" t="s">
-        <v>15</v>
+        <v>28</v>
       </c>
     </row>
     <row r="51" spans="1:11">
       <c r="A51" s="2"/>
       <c r="B51" s="2" t="s">
-        <v>21</v>
+        <v>31</v>
       </c>
       <c r="C51" s="2" t="s">
         <v>92</v>
       </c>
       <c r="D51" s="3" t="s">
-        <v>160</v>
+        <v>194</v>
       </c>
       <c r="E51" t="s">
-        <v>180</v>
+        <v>247</v>
       </c>
       <c r="F51">
         <v>1</v>
       </c>
-      <c r="G51" s="1" t="s">
-        <v>213</v>
-      </c>
       <c r="H51" s="1" t="s">
-        <v>259</v>
+        <v>329</v>
       </c>
       <c r="I51">
         <f>F51*VALUE(LEFT(H51, FIND(":", H51)-1))</f>
         <v>0</v>
       </c>
       <c r="J51" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="K51" t="s">
-        <v>21</v>
+        <v>31</v>
       </c>
     </row>
     <row r="52" spans="1:11">
@@ -3940,26 +4089,26 @@
         <v>93</v>
       </c>
       <c r="D52" s="3" t="s">
-        <v>161</v>
+        <v>195</v>
       </c>
       <c r="E52" t="s">
-        <v>180</v>
+        <v>248</v>
       </c>
       <c r="F52">
         <v>1</v>
       </c>
       <c r="H52" s="1" t="s">
-        <v>272</v>
+        <v>336</v>
       </c>
       <c r="I52">
         <f>F52*VALUE(LEFT(H52, FIND(":", H52)-1))</f>
         <v>0</v>
       </c>
       <c r="J52" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="K52" t="s">
-        <v>21</v>
+        <v>31</v>
       </c>
     </row>
     <row r="53" spans="1:11">
@@ -3969,29 +4118,26 @@
         <v>94</v>
       </c>
       <c r="D53" s="3" t="s">
-        <v>162</v>
+        <v>196</v>
       </c>
       <c r="E53" t="s">
-        <v>180</v>
+        <v>248</v>
       </c>
       <c r="F53">
         <v>1</v>
       </c>
-      <c r="G53" s="1" t="s">
-        <v>214</v>
-      </c>
       <c r="H53" s="1" t="s">
-        <v>266</v>
+        <v>335</v>
       </c>
       <c r="I53">
         <f>F53*VALUE(LEFT(H53, FIND(":", H53)-1))</f>
         <v>0</v>
       </c>
       <c r="J53" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="K53" t="s">
-        <v>21</v>
+        <v>31</v>
       </c>
     </row>
     <row r="54" spans="1:11">
@@ -4001,26 +4147,26 @@
         <v>95</v>
       </c>
       <c r="D54" s="3" t="s">
-        <v>163</v>
+        <v>197</v>
       </c>
       <c r="E54" t="s">
-        <v>180</v>
+        <v>247</v>
       </c>
       <c r="F54">
         <v>1</v>
       </c>
       <c r="H54" s="1" t="s">
-        <v>273</v>
+        <v>329</v>
       </c>
       <c r="I54">
         <f>F54*VALUE(LEFT(H54, FIND(":", H54)-1))</f>
         <v>0</v>
       </c>
       <c r="J54" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="K54" t="s">
-        <v>21</v>
+        <v>31</v>
       </c>
     </row>
     <row r="55" spans="1:11">
@@ -4030,95 +4176,89 @@
         <v>96</v>
       </c>
       <c r="D55" s="3" t="s">
-        <v>164</v>
+        <v>198</v>
       </c>
       <c r="E55" t="s">
-        <v>180</v>
+        <v>247</v>
       </c>
       <c r="F55">
         <v>1</v>
       </c>
-      <c r="G55" s="1" t="s">
-        <v>215</v>
-      </c>
       <c r="H55" s="1" t="s">
-        <v>259</v>
+        <v>329</v>
       </c>
       <c r="I55">
         <f>F55*VALUE(LEFT(H55, FIND(":", H55)-1))</f>
         <v>0</v>
       </c>
       <c r="J55" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="K55" t="s">
-        <v>21</v>
+        <v>31</v>
       </c>
     </row>
     <row r="56" spans="1:11">
       <c r="A56" s="2"/>
-      <c r="B56" s="2" t="s">
-        <v>26</v>
-      </c>
+      <c r="B56" s="2"/>
       <c r="C56" s="2" t="s">
         <v>97</v>
       </c>
       <c r="D56" s="3" t="s">
-        <v>165</v>
+        <v>199</v>
       </c>
       <c r="E56" t="s">
-        <v>179</v>
+        <v>247</v>
       </c>
       <c r="F56">
         <v>1</v>
       </c>
-      <c r="G56" s="1" t="s">
-        <v>216</v>
-      </c>
       <c r="H56" s="1" t="s">
-        <v>259</v>
+        <v>329</v>
       </c>
       <c r="I56">
         <f>F56*VALUE(LEFT(H56, FIND(":", H56)-1))</f>
         <v>0</v>
       </c>
       <c r="J56" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="K56" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
     </row>
     <row r="57" spans="1:11">
       <c r="A57" s="2"/>
-      <c r="B57" s="2"/>
+      <c r="B57" s="2" t="s">
+        <v>11</v>
+      </c>
       <c r="C57" s="2" t="s">
         <v>98</v>
       </c>
       <c r="D57" s="3" t="s">
-        <v>166</v>
+        <v>200</v>
       </c>
       <c r="E57" t="s">
-        <v>179</v>
+        <v>248</v>
       </c>
       <c r="F57">
         <v>1</v>
       </c>
       <c r="G57" s="1" t="s">
-        <v>217</v>
+        <v>268</v>
       </c>
       <c r="H57" s="1" t="s">
-        <v>259</v>
+        <v>328</v>
       </c>
       <c r="I57">
         <f>F57*VALUE(LEFT(H57, FIND(":", H57)-1))</f>
         <v>0</v>
       </c>
       <c r="J57" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="K57" t="s">
-        <v>26</v>
+        <v>11</v>
       </c>
     </row>
     <row r="58" spans="1:11">
@@ -4128,29 +4268,29 @@
         <v>99</v>
       </c>
       <c r="D58" s="3" t="s">
-        <v>167</v>
+        <v>201</v>
       </c>
       <c r="E58" t="s">
-        <v>179</v>
+        <v>248</v>
       </c>
       <c r="F58">
         <v>1</v>
       </c>
       <c r="G58" s="1" t="s">
-        <v>218</v>
+        <v>269</v>
       </c>
       <c r="H58" s="1" t="s">
-        <v>259</v>
+        <v>335</v>
       </c>
       <c r="I58">
         <f>F58*VALUE(LEFT(H58, FIND(":", H58)-1))</f>
         <v>0</v>
       </c>
       <c r="J58" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="K58" t="s">
-        <v>26</v>
+        <v>11</v>
       </c>
     </row>
     <row r="59" spans="1:11">
@@ -4160,29 +4300,29 @@
         <v>100</v>
       </c>
       <c r="D59" s="3" t="s">
-        <v>168</v>
+        <v>202</v>
       </c>
       <c r="E59" t="s">
-        <v>179</v>
+        <v>248</v>
       </c>
       <c r="F59">
         <v>1</v>
       </c>
       <c r="G59" s="1" t="s">
-        <v>219</v>
+        <v>270</v>
       </c>
       <c r="H59" s="1" t="s">
-        <v>259</v>
+        <v>328</v>
       </c>
       <c r="I59">
         <f>F59*VALUE(LEFT(H59, FIND(":", H59)-1))</f>
         <v>0</v>
       </c>
       <c r="J59" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="K59" t="s">
-        <v>26</v>
+        <v>11</v>
       </c>
     </row>
     <row r="60" spans="1:11">
@@ -4192,29 +4332,29 @@
         <v>101</v>
       </c>
       <c r="D60" s="3" t="s">
-        <v>169</v>
+        <v>203</v>
       </c>
       <c r="E60" t="s">
-        <v>180</v>
+        <v>248</v>
       </c>
       <c r="F60">
         <v>1</v>
       </c>
       <c r="G60" s="1" t="s">
-        <v>220</v>
+        <v>271</v>
       </c>
       <c r="H60" s="1" t="s">
-        <v>259</v>
+        <v>335</v>
       </c>
       <c r="I60">
         <f>F60*VALUE(LEFT(H60, FIND(":", H60)-1))</f>
         <v>0</v>
       </c>
       <c r="J60" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="K60" t="s">
-        <v>26</v>
+        <v>11</v>
       </c>
     </row>
     <row r="61" spans="1:11">
@@ -4224,26 +4364,29 @@
         <v>102</v>
       </c>
       <c r="D61" s="3" t="s">
-        <v>170</v>
+        <v>204</v>
       </c>
       <c r="E61" t="s">
-        <v>180</v>
+        <v>248</v>
       </c>
       <c r="F61">
         <v>1</v>
       </c>
+      <c r="G61" s="1" t="s">
+        <v>272</v>
+      </c>
       <c r="H61" s="1" t="s">
-        <v>266</v>
+        <v>335</v>
       </c>
       <c r="I61">
         <f>F61*VALUE(LEFT(H61, FIND(":", H61)-1))</f>
         <v>0</v>
       </c>
       <c r="J61" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="K61" t="s">
-        <v>26</v>
+        <v>11</v>
       </c>
     </row>
     <row r="62" spans="1:11">
@@ -4253,63 +4396,63 @@
         <v>103</v>
       </c>
       <c r="D62" s="3" t="s">
-        <v>171</v>
+        <v>205</v>
       </c>
       <c r="E62" t="s">
-        <v>179</v>
+        <v>248</v>
       </c>
       <c r="F62">
         <v>1</v>
       </c>
       <c r="G62" s="1" t="s">
-        <v>221</v>
+        <v>273</v>
       </c>
       <c r="H62" s="1" t="s">
-        <v>259</v>
+        <v>328</v>
       </c>
       <c r="I62">
         <f>F62*VALUE(LEFT(H62, FIND(":", H62)-1))</f>
         <v>0</v>
       </c>
       <c r="J62" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="K62" t="s">
-        <v>26</v>
+        <v>11</v>
       </c>
     </row>
     <row r="63" spans="1:11">
       <c r="A63" s="2"/>
       <c r="B63" s="2" t="s">
-        <v>30</v>
+        <v>12</v>
       </c>
       <c r="C63" s="2" t="s">
         <v>104</v>
       </c>
       <c r="D63" s="3" t="s">
-        <v>172</v>
+        <v>206</v>
       </c>
       <c r="E63" t="s">
-        <v>180</v>
+        <v>248</v>
       </c>
       <c r="F63">
         <v>1</v>
       </c>
       <c r="G63" s="1" t="s">
-        <v>222</v>
+        <v>274</v>
       </c>
       <c r="H63" s="1" t="s">
-        <v>259</v>
+        <v>328</v>
       </c>
       <c r="I63">
         <f>F63*VALUE(LEFT(H63, FIND(":", H63)-1))</f>
         <v>0</v>
       </c>
       <c r="J63" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="K63" t="s">
-        <v>30</v>
+        <v>12</v>
       </c>
     </row>
     <row r="64" spans="1:11">
@@ -4319,29 +4462,29 @@
         <v>105</v>
       </c>
       <c r="D64" s="3" t="s">
-        <v>173</v>
+        <v>207</v>
       </c>
       <c r="E64" t="s">
-        <v>179</v>
+        <v>248</v>
       </c>
       <c r="F64">
         <v>1</v>
       </c>
       <c r="G64" s="1" t="s">
-        <v>223</v>
+        <v>275</v>
       </c>
       <c r="H64" s="1" t="s">
-        <v>259</v>
+        <v>328</v>
       </c>
       <c r="I64">
         <f>F64*VALUE(LEFT(H64, FIND(":", H64)-1))</f>
         <v>0</v>
       </c>
       <c r="J64" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="K64" t="s">
-        <v>30</v>
+        <v>12</v>
       </c>
     </row>
     <row r="65" spans="1:11">
@@ -4351,29 +4494,26 @@
         <v>106</v>
       </c>
       <c r="D65" s="3" t="s">
-        <v>174</v>
+        <v>208</v>
       </c>
       <c r="E65" t="s">
-        <v>179</v>
+        <v>248</v>
       </c>
       <c r="F65">
         <v>1</v>
       </c>
-      <c r="G65" s="1" t="s">
-        <v>224</v>
-      </c>
       <c r="H65" s="1" t="s">
-        <v>259</v>
+        <v>337</v>
       </c>
       <c r="I65">
         <f>F65*VALUE(LEFT(H65, FIND(":", H65)-1))</f>
         <v>0</v>
       </c>
       <c r="J65" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="K65" t="s">
-        <v>30</v>
+        <v>12</v>
       </c>
     </row>
     <row r="66" spans="1:11">
@@ -4383,61 +4523,60 @@
         <v>107</v>
       </c>
       <c r="D66" s="3" t="s">
-        <v>175</v>
+        <v>209</v>
       </c>
       <c r="E66" t="s">
-        <v>179</v>
+        <v>248</v>
       </c>
       <c r="F66">
         <v>1</v>
       </c>
       <c r="G66" s="1" t="s">
-        <v>225</v>
+        <v>276</v>
       </c>
       <c r="H66" s="1" t="s">
-        <v>259</v>
+        <v>328</v>
       </c>
       <c r="I66">
         <f>F66*VALUE(LEFT(H66, FIND(":", H66)-1))</f>
         <v>0</v>
       </c>
       <c r="J66" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="K66" t="s">
-        <v>30</v>
+        <v>12</v>
       </c>
     </row>
     <row r="67" spans="1:11">
       <c r="A67" s="2"/>
-      <c r="B67" s="2"/>
+      <c r="B67" s="2" t="s">
+        <v>16</v>
+      </c>
       <c r="C67" s="2" t="s">
         <v>108</v>
       </c>
       <c r="D67" s="3" t="s">
-        <v>176</v>
+        <v>210</v>
       </c>
       <c r="E67" t="s">
-        <v>179</v>
+        <v>248</v>
       </c>
       <c r="F67">
         <v>1</v>
       </c>
-      <c r="G67" s="1" t="s">
-        <v>226</v>
-      </c>
       <c r="H67" s="1" t="s">
-        <v>259</v>
+        <v>338</v>
       </c>
       <c r="I67">
         <f>F67*VALUE(LEFT(H67, FIND(":", H67)-1))</f>
         <v>0</v>
       </c>
       <c r="J67" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="K67" t="s">
-        <v>30</v>
+        <v>16</v>
       </c>
     </row>
     <row r="68" spans="1:11">
@@ -4447,84 +4586,1140 @@
         <v>109</v>
       </c>
       <c r="D68" s="3" t="s">
-        <v>177</v>
+        <v>211</v>
       </c>
       <c r="E68" t="s">
-        <v>180</v>
+        <v>248</v>
       </c>
       <c r="F68">
         <v>1</v>
       </c>
+      <c r="G68" s="1" t="s">
+        <v>277</v>
+      </c>
       <c r="H68" s="1" t="s">
-        <v>272</v>
+        <v>328</v>
       </c>
       <c r="I68">
         <f>F68*VALUE(LEFT(H68, FIND(":", H68)-1))</f>
         <v>0</v>
       </c>
       <c r="J68" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="K68" t="s">
-        <v>30</v>
+        <v>16</v>
       </c>
     </row>
     <row r="69" spans="1:11">
-      <c r="A69" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="B69" s="2" t="s">
-        <v>27</v>
-      </c>
+      <c r="A69" s="2"/>
+      <c r="B69" s="2"/>
       <c r="C69" s="2" t="s">
         <v>110</v>
       </c>
       <c r="D69" s="3" t="s">
-        <v>178</v>
+        <v>212</v>
       </c>
       <c r="E69" t="s">
-        <v>180</v>
+        <v>248</v>
       </c>
       <c r="F69">
         <v>1</v>
       </c>
+      <c r="G69" s="1" t="s">
+        <v>278</v>
+      </c>
       <c r="H69" s="1" t="s">
-        <v>274</v>
+        <v>328</v>
       </c>
       <c r="I69">
         <f>F69*VALUE(LEFT(H69, FIND(":", H69)-1))</f>
         <v>0</v>
       </c>
       <c r="J69" t="s">
+        <v>9</v>
+      </c>
+      <c r="K69" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="70" spans="1:11">
+      <c r="A70" s="2"/>
+      <c r="B70" s="2"/>
+      <c r="C70" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="D70" s="3" t="s">
+        <v>213</v>
+      </c>
+      <c r="E70" t="s">
+        <v>250</v>
+      </c>
+      <c r="F70">
+        <v>1</v>
+      </c>
+      <c r="H70" s="1" t="s">
+        <v>338</v>
+      </c>
+      <c r="I70">
+        <f>F70*VALUE(LEFT(H70, FIND(":", H70)-1))</f>
+        <v>0</v>
+      </c>
+      <c r="J70" t="s">
+        <v>9</v>
+      </c>
+      <c r="K70" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="71" spans="1:11">
+      <c r="A71" s="2"/>
+      <c r="B71" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="C71" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="D71" s="3" t="s">
+        <v>214</v>
+      </c>
+      <c r="E71" t="s">
+        <v>247</v>
+      </c>
+      <c r="F71">
+        <v>1</v>
+      </c>
+      <c r="H71" s="1" t="s">
+        <v>329</v>
+      </c>
+      <c r="I71">
+        <f>F71*VALUE(LEFT(H71, FIND(":", H71)-1))</f>
+        <v>0</v>
+      </c>
+      <c r="J71" t="s">
+        <v>9</v>
+      </c>
+      <c r="K71" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="72" spans="1:11">
+      <c r="A72" s="2"/>
+      <c r="B72" s="2"/>
+      <c r="C72" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="D72" s="3" t="s">
+        <v>215</v>
+      </c>
+      <c r="E72" t="s">
+        <v>248</v>
+      </c>
+      <c r="F72">
+        <v>1</v>
+      </c>
+      <c r="G72" s="1" t="s">
+        <v>279</v>
+      </c>
+      <c r="H72" s="1" t="s">
+        <v>328</v>
+      </c>
+      <c r="I72">
+        <f>F72*VALUE(LEFT(H72, FIND(":", H72)-1))</f>
+        <v>0</v>
+      </c>
+      <c r="J72" t="s">
+        <v>9</v>
+      </c>
+      <c r="K72" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="73" spans="1:11">
+      <c r="A73" s="2"/>
+      <c r="B73" s="2"/>
+      <c r="C73" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="D73" s="3" t="s">
+        <v>216</v>
+      </c>
+      <c r="E73" t="s">
+        <v>248</v>
+      </c>
+      <c r="F73">
+        <v>1</v>
+      </c>
+      <c r="G73" s="1" t="s">
+        <v>280</v>
+      </c>
+      <c r="H73" s="1" t="s">
+        <v>328</v>
+      </c>
+      <c r="I73">
+        <f>F73*VALUE(LEFT(H73, FIND(":", H73)-1))</f>
+        <v>0</v>
+      </c>
+      <c r="J73" t="s">
+        <v>9</v>
+      </c>
+      <c r="K73" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="74" spans="1:11">
+      <c r="A74" s="2"/>
+      <c r="B74" s="2"/>
+      <c r="C74" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="D74" s="3" t="s">
+        <v>217</v>
+      </c>
+      <c r="E74" t="s">
+        <v>247</v>
+      </c>
+      <c r="F74">
+        <v>1</v>
+      </c>
+      <c r="H74" s="1" t="s">
+        <v>329</v>
+      </c>
+      <c r="I74">
+        <f>F74*VALUE(LEFT(H74, FIND(":", H74)-1))</f>
+        <v>0</v>
+      </c>
+      <c r="J74" t="s">
+        <v>9</v>
+      </c>
+      <c r="K74" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="75" spans="1:11">
+      <c r="A75" s="2"/>
+      <c r="B75" s="2"/>
+      <c r="C75" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="D75" s="3" t="s">
+        <v>218</v>
+      </c>
+      <c r="E75" t="s">
+        <v>248</v>
+      </c>
+      <c r="F75">
+        <v>1</v>
+      </c>
+      <c r="H75" s="1" t="s">
+        <v>339</v>
+      </c>
+      <c r="I75">
+        <f>F75*VALUE(LEFT(H75, FIND(":", H75)-1))</f>
+        <v>0</v>
+      </c>
+      <c r="J75" t="s">
+        <v>9</v>
+      </c>
+      <c r="K75" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="76" spans="1:11">
+      <c r="A76" s="2"/>
+      <c r="B76" s="2"/>
+      <c r="C76" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="D76" s="3" t="s">
+        <v>219</v>
+      </c>
+      <c r="E76" t="s">
+        <v>247</v>
+      </c>
+      <c r="F76">
+        <v>1</v>
+      </c>
+      <c r="H76" s="1" t="s">
+        <v>329</v>
+      </c>
+      <c r="I76">
+        <f>F76*VALUE(LEFT(H76, FIND(":", H76)-1))</f>
+        <v>0</v>
+      </c>
+      <c r="J76" t="s">
+        <v>9</v>
+      </c>
+      <c r="K76" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="77" spans="1:11">
+      <c r="A77" s="2"/>
+      <c r="B77" s="2"/>
+      <c r="C77" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="D77" s="3" t="s">
+        <v>220</v>
+      </c>
+      <c r="E77" t="s">
+        <v>247</v>
+      </c>
+      <c r="F77">
+        <v>1</v>
+      </c>
+      <c r="H77" s="1" t="s">
+        <v>329</v>
+      </c>
+      <c r="I77">
+        <f>F77*VALUE(LEFT(H77, FIND(":", H77)-1))</f>
+        <v>0</v>
+      </c>
+      <c r="J77" t="s">
+        <v>9</v>
+      </c>
+      <c r="K77" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="78" spans="1:11">
+      <c r="A78" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B78" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C78" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="D78" s="3" t="s">
+        <v>221</v>
+      </c>
+      <c r="E78" t="s">
+        <v>248</v>
+      </c>
+      <c r="F78">
+        <v>1</v>
+      </c>
+      <c r="H78" s="1" t="s">
+        <v>340</v>
+      </c>
+      <c r="I78">
+        <f>F78*VALUE(LEFT(H78, FIND(":", H78)-1))</f>
+        <v>0</v>
+      </c>
+      <c r="J78" t="s">
+        <v>8</v>
+      </c>
+      <c r="K78" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="79" spans="1:11">
+      <c r="A79" s="2"/>
+      <c r="B79" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C79" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="D79" s="3" t="s">
+        <v>222</v>
+      </c>
+      <c r="E79" t="s">
+        <v>248</v>
+      </c>
+      <c r="F79">
+        <v>1</v>
+      </c>
+      <c r="H79" s="1" t="s">
+        <v>333</v>
+      </c>
+      <c r="I79">
+        <f>F79*VALUE(LEFT(H79, FIND(":", H79)-1))</f>
+        <v>0</v>
+      </c>
+      <c r="J79" t="s">
+        <v>8</v>
+      </c>
+      <c r="K79" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="80" spans="1:11">
+      <c r="A80" s="2"/>
+      <c r="B80" s="2"/>
+      <c r="C80" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="D80" s="3" t="s">
+        <v>223</v>
+      </c>
+      <c r="E80" t="s">
+        <v>248</v>
+      </c>
+      <c r="F80">
+        <v>1</v>
+      </c>
+      <c r="H80" s="1" t="s">
+        <v>333</v>
+      </c>
+      <c r="I80">
+        <f>F80*VALUE(LEFT(H80, FIND(":", H80)-1))</f>
+        <v>0</v>
+      </c>
+      <c r="J80" t="s">
+        <v>8</v>
+      </c>
+      <c r="K80" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="81" spans="1:11">
+      <c r="A81" s="2"/>
+      <c r="B81" s="2"/>
+      <c r="C81" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="D81" s="3" t="s">
+        <v>224</v>
+      </c>
+      <c r="E81" t="s">
+        <v>247</v>
+      </c>
+      <c r="F81">
+        <v>1</v>
+      </c>
+      <c r="H81" s="1" t="s">
+        <v>329</v>
+      </c>
+      <c r="I81">
+        <f>F81*VALUE(LEFT(H81, FIND(":", H81)-1))</f>
+        <v>0</v>
+      </c>
+      <c r="J81" t="s">
+        <v>8</v>
+      </c>
+      <c r="K81" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="82" spans="1:11">
+      <c r="A82" s="2"/>
+      <c r="B82" s="2"/>
+      <c r="C82" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="D82" s="3" t="s">
+        <v>225</v>
+      </c>
+      <c r="E82" t="s">
+        <v>247</v>
+      </c>
+      <c r="F82">
+        <v>1</v>
+      </c>
+      <c r="H82" s="1" t="s">
+        <v>329</v>
+      </c>
+      <c r="I82">
+        <f>F82*VALUE(LEFT(H82, FIND(":", H82)-1))</f>
+        <v>0</v>
+      </c>
+      <c r="J82" t="s">
+        <v>8</v>
+      </c>
+      <c r="K82" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="83" spans="1:11">
+      <c r="A83" s="2"/>
+      <c r="B83" s="2"/>
+      <c r="C83" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="D83" s="3" t="s">
+        <v>226</v>
+      </c>
+      <c r="E83" t="s">
+        <v>247</v>
+      </c>
+      <c r="F83">
+        <v>1</v>
+      </c>
+      <c r="H83" s="1" t="s">
+        <v>329</v>
+      </c>
+      <c r="I83">
+        <f>F83*VALUE(LEFT(H83, FIND(":", H83)-1))</f>
+        <v>0</v>
+      </c>
+      <c r="J83" t="s">
+        <v>8</v>
+      </c>
+      <c r="K83" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="84" spans="1:11">
+      <c r="A84" s="2"/>
+      <c r="B84" s="2"/>
+      <c r="C84" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="D84" s="3" t="s">
+        <v>227</v>
+      </c>
+      <c r="E84" t="s">
+        <v>247</v>
+      </c>
+      <c r="F84">
+        <v>1</v>
+      </c>
+      <c r="H84" s="1" t="s">
+        <v>329</v>
+      </c>
+      <c r="I84">
+        <f>F84*VALUE(LEFT(H84, FIND(":", H84)-1))</f>
+        <v>0</v>
+      </c>
+      <c r="J84" t="s">
+        <v>8</v>
+      </c>
+      <c r="K84" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="85" spans="1:11">
+      <c r="A85" s="2"/>
+      <c r="B85" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C85" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="D85" s="3" t="s">
+        <v>228</v>
+      </c>
+      <c r="E85" t="s">
+        <v>248</v>
+      </c>
+      <c r="F85">
+        <v>1</v>
+      </c>
+      <c r="G85" s="1" t="s">
+        <v>281</v>
+      </c>
+      <c r="H85" s="1" t="s">
+        <v>328</v>
+      </c>
+      <c r="I85">
+        <f>F85*VALUE(LEFT(H85, FIND(":", H85)-1))</f>
+        <v>0</v>
+      </c>
+      <c r="J85" t="s">
+        <v>8</v>
+      </c>
+      <c r="K85" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="86" spans="1:11">
+      <c r="A86" s="2"/>
+      <c r="B86" s="2"/>
+      <c r="C86" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="D86" s="3" t="s">
+        <v>229</v>
+      </c>
+      <c r="E86" t="s">
+        <v>248</v>
+      </c>
+      <c r="F86">
+        <v>1</v>
+      </c>
+      <c r="H86" s="1" t="s">
+        <v>341</v>
+      </c>
+      <c r="I86">
+        <f>F86*VALUE(LEFT(H86, FIND(":", H86)-1))</f>
+        <v>0</v>
+      </c>
+      <c r="J86" t="s">
+        <v>8</v>
+      </c>
+      <c r="K86" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="87" spans="1:11">
+      <c r="A87" s="2"/>
+      <c r="B87" s="2"/>
+      <c r="C87" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="D87" s="3" t="s">
+        <v>230</v>
+      </c>
+      <c r="E87" t="s">
+        <v>248</v>
+      </c>
+      <c r="F87">
+        <v>1</v>
+      </c>
+      <c r="G87" s="1" t="s">
+        <v>282</v>
+      </c>
+      <c r="H87" s="1" t="s">
+        <v>335</v>
+      </c>
+      <c r="I87">
+        <f>F87*VALUE(LEFT(H87, FIND(":", H87)-1))</f>
+        <v>0</v>
+      </c>
+      <c r="J87" t="s">
+        <v>8</v>
+      </c>
+      <c r="K87" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="88" spans="1:11">
+      <c r="A88" s="2"/>
+      <c r="B88" s="2"/>
+      <c r="C88" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="D88" s="3" t="s">
+        <v>231</v>
+      </c>
+      <c r="E88" t="s">
+        <v>248</v>
+      </c>
+      <c r="F88">
+        <v>1</v>
+      </c>
+      <c r="H88" s="1" t="s">
+        <v>342</v>
+      </c>
+      <c r="I88">
+        <f>F88*VALUE(LEFT(H88, FIND(":", H88)-1))</f>
+        <v>0</v>
+      </c>
+      <c r="J88" t="s">
+        <v>8</v>
+      </c>
+      <c r="K88" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="89" spans="1:11">
+      <c r="A89" s="2"/>
+      <c r="B89" s="2"/>
+      <c r="C89" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="D89" s="3" t="s">
+        <v>232</v>
+      </c>
+      <c r="E89" t="s">
+        <v>248</v>
+      </c>
+      <c r="F89">
+        <v>1</v>
+      </c>
+      <c r="G89" s="1" t="s">
+        <v>283</v>
+      </c>
+      <c r="H89" s="1" t="s">
+        <v>328</v>
+      </c>
+      <c r="I89">
+        <f>F89*VALUE(LEFT(H89, FIND(":", H89)-1))</f>
+        <v>0</v>
+      </c>
+      <c r="J89" t="s">
+        <v>8</v>
+      </c>
+      <c r="K89" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="90" spans="1:11">
+      <c r="A90" s="2"/>
+      <c r="B90" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="C90" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="D90" s="3" t="s">
+        <v>233</v>
+      </c>
+      <c r="E90" t="s">
+        <v>247</v>
+      </c>
+      <c r="F90">
+        <v>1</v>
+      </c>
+      <c r="G90" s="1" t="s">
+        <v>284</v>
+      </c>
+      <c r="H90" s="1" t="s">
+        <v>328</v>
+      </c>
+      <c r="I90">
+        <f>F90*VALUE(LEFT(H90, FIND(":", H90)-1))</f>
+        <v>0</v>
+      </c>
+      <c r="J90" t="s">
+        <v>8</v>
+      </c>
+      <c r="K90" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="91" spans="1:11">
+      <c r="A91" s="2"/>
+      <c r="B91" s="2"/>
+      <c r="C91" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="D91" s="3" t="s">
+        <v>234</v>
+      </c>
+      <c r="E91" t="s">
+        <v>247</v>
+      </c>
+      <c r="F91">
+        <v>1</v>
+      </c>
+      <c r="G91" s="1" t="s">
+        <v>285</v>
+      </c>
+      <c r="H91" s="1" t="s">
+        <v>328</v>
+      </c>
+      <c r="I91">
+        <f>F91*VALUE(LEFT(H91, FIND(":", H91)-1))</f>
+        <v>0</v>
+      </c>
+      <c r="J91" t="s">
+        <v>8</v>
+      </c>
+      <c r="K91" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="92" spans="1:11">
+      <c r="A92" s="2"/>
+      <c r="B92" s="2"/>
+      <c r="C92" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="D92" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="E92" t="s">
+        <v>247</v>
+      </c>
+      <c r="F92">
+        <v>1</v>
+      </c>
+      <c r="G92" s="1" t="s">
+        <v>286</v>
+      </c>
+      <c r="H92" s="1" t="s">
+        <v>328</v>
+      </c>
+      <c r="I92">
+        <f>F92*VALUE(LEFT(H92, FIND(":", H92)-1))</f>
+        <v>0</v>
+      </c>
+      <c r="J92" t="s">
+        <v>8</v>
+      </c>
+      <c r="K92" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="93" spans="1:11">
+      <c r="A93" s="2"/>
+      <c r="B93" s="2"/>
+      <c r="C93" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="D93" s="3" t="s">
+        <v>236</v>
+      </c>
+      <c r="E93" t="s">
+        <v>247</v>
+      </c>
+      <c r="F93">
+        <v>1</v>
+      </c>
+      <c r="G93" s="1" t="s">
+        <v>287</v>
+      </c>
+      <c r="H93" s="1" t="s">
+        <v>328</v>
+      </c>
+      <c r="I93">
+        <f>F93*VALUE(LEFT(H93, FIND(":", H93)-1))</f>
+        <v>0</v>
+      </c>
+      <c r="J93" t="s">
+        <v>8</v>
+      </c>
+      <c r="K93" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="94" spans="1:11">
+      <c r="A94" s="2"/>
+      <c r="B94" s="2"/>
+      <c r="C94" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="D94" s="3" t="s">
+        <v>237</v>
+      </c>
+      <c r="E94" t="s">
+        <v>248</v>
+      </c>
+      <c r="F94">
+        <v>1</v>
+      </c>
+      <c r="G94" s="1" t="s">
+        <v>288</v>
+      </c>
+      <c r="H94" s="1" t="s">
+        <v>328</v>
+      </c>
+      <c r="I94">
+        <f>F94*VALUE(LEFT(H94, FIND(":", H94)-1))</f>
+        <v>0</v>
+      </c>
+      <c r="J94" t="s">
+        <v>8</v>
+      </c>
+      <c r="K94" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="95" spans="1:11">
+      <c r="A95" s="2"/>
+      <c r="B95" s="2"/>
+      <c r="C95" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="D95" s="3" t="s">
+        <v>238</v>
+      </c>
+      <c r="E95" t="s">
+        <v>248</v>
+      </c>
+      <c r="F95">
+        <v>1</v>
+      </c>
+      <c r="H95" s="1" t="s">
+        <v>335</v>
+      </c>
+      <c r="I95">
+        <f>F95*VALUE(LEFT(H95, FIND(":", H95)-1))</f>
+        <v>0</v>
+      </c>
+      <c r="J95" t="s">
+        <v>8</v>
+      </c>
+      <c r="K95" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="96" spans="1:11">
+      <c r="A96" s="2"/>
+      <c r="B96" s="2"/>
+      <c r="C96" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="D96" s="3" t="s">
+        <v>239</v>
+      </c>
+      <c r="E96" t="s">
+        <v>247</v>
+      </c>
+      <c r="F96">
+        <v>1</v>
+      </c>
+      <c r="G96" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="H96" s="1" t="s">
+        <v>328</v>
+      </c>
+      <c r="I96">
+        <f>F96*VALUE(LEFT(H96, FIND(":", H96)-1))</f>
+        <v>0</v>
+      </c>
+      <c r="J96" t="s">
+        <v>8</v>
+      </c>
+      <c r="K96" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="97" spans="1:11">
+      <c r="A97" s="2"/>
+      <c r="B97" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="C97" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="D97" s="3" t="s">
+        <v>240</v>
+      </c>
+      <c r="E97" t="s">
+        <v>248</v>
+      </c>
+      <c r="F97">
+        <v>1</v>
+      </c>
+      <c r="G97" s="1" t="s">
+        <v>290</v>
+      </c>
+      <c r="H97" s="1" t="s">
+        <v>328</v>
+      </c>
+      <c r="I97">
+        <f>F97*VALUE(LEFT(H97, FIND(":", H97)-1))</f>
+        <v>0</v>
+      </c>
+      <c r="J97" t="s">
+        <v>8</v>
+      </c>
+      <c r="K97" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="98" spans="1:11">
+      <c r="A98" s="2"/>
+      <c r="B98" s="2"/>
+      <c r="C98" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="D98" s="3" t="s">
+        <v>241</v>
+      </c>
+      <c r="E98" t="s">
+        <v>247</v>
+      </c>
+      <c r="F98">
+        <v>1</v>
+      </c>
+      <c r="G98" s="1" t="s">
+        <v>291</v>
+      </c>
+      <c r="H98" s="1" t="s">
+        <v>328</v>
+      </c>
+      <c r="I98">
+        <f>F98*VALUE(LEFT(H98, FIND(":", H98)-1))</f>
+        <v>0</v>
+      </c>
+      <c r="J98" t="s">
+        <v>8</v>
+      </c>
+      <c r="K98" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="99" spans="1:11">
+      <c r="A99" s="2"/>
+      <c r="B99" s="2"/>
+      <c r="C99" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="D99" s="3" t="s">
+        <v>242</v>
+      </c>
+      <c r="E99" t="s">
+        <v>247</v>
+      </c>
+      <c r="F99">
+        <v>1</v>
+      </c>
+      <c r="G99" s="1" t="s">
+        <v>292</v>
+      </c>
+      <c r="H99" s="1" t="s">
+        <v>328</v>
+      </c>
+      <c r="I99">
+        <f>F99*VALUE(LEFT(H99, FIND(":", H99)-1))</f>
+        <v>0</v>
+      </c>
+      <c r="J99" t="s">
+        <v>8</v>
+      </c>
+      <c r="K99" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="100" spans="1:11">
+      <c r="A100" s="2"/>
+      <c r="B100" s="2"/>
+      <c r="C100" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="D100" s="3" t="s">
+        <v>243</v>
+      </c>
+      <c r="E100" t="s">
+        <v>247</v>
+      </c>
+      <c r="F100">
+        <v>1</v>
+      </c>
+      <c r="G100" s="1" t="s">
+        <v>293</v>
+      </c>
+      <c r="H100" s="1" t="s">
+        <v>328</v>
+      </c>
+      <c r="I100">
+        <f>F100*VALUE(LEFT(H100, FIND(":", H100)-1))</f>
+        <v>0</v>
+      </c>
+      <c r="J100" t="s">
+        <v>8</v>
+      </c>
+      <c r="K100" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="101" spans="1:11">
+      <c r="A101" s="2"/>
+      <c r="B101" s="2"/>
+      <c r="C101" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="D101" s="3" t="s">
+        <v>244</v>
+      </c>
+      <c r="E101" t="s">
+        <v>247</v>
+      </c>
+      <c r="F101">
+        <v>1</v>
+      </c>
+      <c r="G101" s="1" t="s">
+        <v>294</v>
+      </c>
+      <c r="H101" s="1" t="s">
+        <v>328</v>
+      </c>
+      <c r="I101">
+        <f>F101*VALUE(LEFT(H101, FIND(":", H101)-1))</f>
+        <v>0</v>
+      </c>
+      <c r="J101" t="s">
+        <v>8</v>
+      </c>
+      <c r="K101" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="102" spans="1:11">
+      <c r="A102" s="2"/>
+      <c r="B102" s="2"/>
+      <c r="C102" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="D102" s="3" t="s">
+        <v>245</v>
+      </c>
+      <c r="E102" t="s">
+        <v>248</v>
+      </c>
+      <c r="F102">
+        <v>1</v>
+      </c>
+      <c r="H102" s="1" t="s">
+        <v>341</v>
+      </c>
+      <c r="I102">
+        <f>F102*VALUE(LEFT(H102, FIND(":", H102)-1))</f>
+        <v>0</v>
+      </c>
+      <c r="J102" t="s">
+        <v>8</v>
+      </c>
+      <c r="K102" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="103" spans="1:11">
+      <c r="A103" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="K69" t="s">
+      <c r="B103" s="2" t="s">
         <v>27</v>
       </c>
+      <c r="C103" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="D103" s="3" t="s">
+        <v>246</v>
+      </c>
+      <c r="E103" t="s">
+        <v>248</v>
+      </c>
+      <c r="F103">
+        <v>1</v>
+      </c>
+      <c r="H103" s="1" t="s">
+        <v>343</v>
+      </c>
+      <c r="I103">
+        <f>F103*VALUE(LEFT(H103, FIND(":", H103)-1))</f>
+        <v>0</v>
+      </c>
+      <c r="J103" t="s">
+        <v>6</v>
+      </c>
+      <c r="K103" t="s">
+        <v>27</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="19">
-    <mergeCell ref="A2:A19"/>
-    <mergeCell ref="A20:A47"/>
-    <mergeCell ref="A48:A68"/>
+  <mergeCells count="21">
+    <mergeCell ref="A2:A32"/>
+    <mergeCell ref="A33:A77"/>
+    <mergeCell ref="A78:A102"/>
     <mergeCell ref="B2:B5"/>
-    <mergeCell ref="B8:B10"/>
+    <mergeCell ref="B6:B10"/>
     <mergeCell ref="B11:B16"/>
-    <mergeCell ref="B17:B18"/>
-    <mergeCell ref="B20:B23"/>
-    <mergeCell ref="B24:B25"/>
-    <mergeCell ref="B26:B28"/>
-    <mergeCell ref="B29:B30"/>
-    <mergeCell ref="B31:B36"/>
-    <mergeCell ref="B37:B40"/>
-    <mergeCell ref="B41:B44"/>
-    <mergeCell ref="B45:B47"/>
-    <mergeCell ref="B49:B50"/>
-    <mergeCell ref="B51:B55"/>
-    <mergeCell ref="B56:B62"/>
-    <mergeCell ref="B63:B68"/>
+    <mergeCell ref="B17:B19"/>
+    <mergeCell ref="B20:B25"/>
+    <mergeCell ref="B26:B31"/>
+    <mergeCell ref="B33:B41"/>
+    <mergeCell ref="B42:B47"/>
+    <mergeCell ref="B48:B50"/>
+    <mergeCell ref="B51:B56"/>
+    <mergeCell ref="B57:B62"/>
+    <mergeCell ref="B63:B66"/>
+    <mergeCell ref="B67:B70"/>
+    <mergeCell ref="B71:B77"/>
+    <mergeCell ref="B79:B84"/>
+    <mergeCell ref="B85:B89"/>
+    <mergeCell ref="B90:B96"/>
+    <mergeCell ref="B97:B102"/>
   </mergeCells>
-  <dataValidations count="68">
+  <dataValidations count="102">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H2">
       <formula1>"0: 0 items completed,3: 1 item completed,5: 2 items completed,8: 3 items completed,10: 4 items completed"</formula1>
     </dataValidation>
@@ -4538,169 +5733,169 @@
       <formula1>"0: No items completed,3: item 1 completed,5: items 1-2 completed,8: items 1-3 completed,10: items 1-4 completed"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H6">
+      <formula1>"0: Not done,10: Completed"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H7">
+      <formula1>"0: Not done,10: Completed"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H8">
+      <formula1>"0: Not done,10: Completed"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H9">
       <formula1>"0: No items completed,5: 1 item completed,10: 2 items completed"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H7">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H10">
+      <formula1>"0: Not done,10: Completed"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H11">
       <formula1>"0: Not done,10: Defined"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H8">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H12">
+      <formula1>"0: Not done,10: Completed"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H13">
+      <formula1>"0: Not done,10: Completed"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H14">
+      <formula1>"0: Not done,10: Completed"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H15">
+      <formula1>"0: Not done,10: Completed"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H16">
+      <formula1>"0: Not done,10: Completed"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H17">
       <formula1>"0: Low Maturity. Score Range (0-8),4: Developing. Score Range (9-17),7: Established. Score Range (18-24),10: Optimizing. Score Range (25-29)"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H9">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H18">
       <formula1>"0: Low Maturity. Score Range (0-15),4: Developing. Score Range (16-31),7: Established. Score Range (32-44),10: Optimizing. Score Range (45-52)"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H10">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H19">
       <formula1>"0: No items completed,2: 1 item completed,4: 2 items completed,6: 3 items completed,8: 4 items completed,10: 5 items completed"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H11">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H20">
       <formula1>"0: No items completed,2: item 1 completed,4: items 1-2 completed,6: items 1-3 completed,8: items 1-4 completed,10: items 1-5 completed"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H12">
-      <formula1>"0: No items completed,2: 1 item completed,4: 2 items completed,6: 3 items completed,8: 4 items completed,10: 5 items completed"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H13">
-      <formula1>"0: No items completed,4: 1 item completed,7: 2 items completed,10: 3 items completed"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H14">
-      <formula1>"0: No items completed,4: 1 item completed,7: 2 items completed,10: 3 items completed"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H15">
-      <formula1>"0: No items completed,3: item 1 completed,5: items 1-2 completed,8: items 1-3 completed,10: items 1-4 completed"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H16">
-      <formula1>"0: No items completed,4: 1 item completed,7: 2 items completed,10: 3 items completed"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H17">
-      <formula1>"0: Not done,10: Done and clearly defined"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H18">
-      <formula1>"0: Not done,10: Defined"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H19">
-      <formula1>"0: No executive sponsor identified,10: Executive sponsor formally identified and actively engaged"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H20">
-      <formula1>"0: Does not exist,10: Exists"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H21">
       <formula1>"0: No items completed,2: 1 item completed,4: 2 items completed,6: 3 items completed,8: 4 items completed,10: 5 items completed"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H22">
-      <formula1>"0: No documented method,10: Documented method of assessing modernization efforts"</formula1>
+      <formula1>"0: No items completed,4: 1 item completed,7: 2 items completed,10: 3 items completed"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H23">
       <formula1>"0: No items completed,4: 1 item completed,7: 2 items completed,10: 3 items completed"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H24">
+      <formula1>"0: No items completed,3: item 1 completed,5: items 1-2 completed,8: items 1-3 completed,10: items 1-4 completed"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H25">
+      <formula1>"0: No items completed,4: 1 item completed,7: 2 items completed,10: 3 items completed"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H26">
+      <formula1>"0: Not done,10: Completed"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H27">
+      <formula1>"0: Not done,10: Completed"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H28">
+      <formula1>"0: Not done,10: Done and clearly defined"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H29">
+      <formula1>"0: Not done,10: Completed"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H30">
+      <formula1>"0: Not done,10: Completed"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H31">
+      <formula1>"0: Not done,10: Defined"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H32">
+      <formula1>"0: No executive sponsor identified,10: Executive sponsor formally identified and actively engaged"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H33">
+      <formula1>"0: Does not exist,10: Exists"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H34">
+      <formula1>"0: No items completed,2: 1 item completed,4: 2 items completed,6: 3 items completed,8: 4 items completed,10: 5 items completed"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H35">
+      <formula1>"0: No documented method,10: Documented method of assessing modernization efforts"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H36">
+      <formula1>"0: Not done,10: Completed"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H37">
+      <formula1>"0: Not done,10: Completed"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H38">
+      <formula1>"0: No items completed,4: 1 item completed,7: 2 items completed,10: 3 items completed"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H39">
+      <formula1>"0: Not done,10: Completed"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H40">
+      <formula1>"0: Not done,10: Completed"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H41">
+      <formula1>"0: Not done,10: Completed"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H42">
       <formula1>"0: 0%,1: 10%,2: 20%,3: 30%,4: 40%,5: 50%,6: 60%,7: 70%,8: 80%,9: 90%,10: Near 100%"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H25">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H43">
+      <formula1>"0: Not done,10: Completed"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H44">
+      <formula1>"0: Not done,10: Completed"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H45">
       <formula1>"0: Not done,10: Policy in place and published"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H26">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H46">
+      <formula1>"0: Not done,10: Completed"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H47">
+      <formula1>"0: Not done,10: Completed"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H48">
       <formula1>"0: Not done,10: Policy in place and published"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H27">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H49">
       <formula1>"0: Not done,10: Policy in place and published"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H28">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H50">
       <formula1>"0: No items completed,2: 1 item completed,4: 2 items completed,6: 3 items completed,8: 4 items completed,10: 5 items completed"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H29">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H51">
+      <formula1>"0: Not done,10: Completed"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H52">
       <formula1>"0: No teardown/shutdown policy,3: Published policy,6: Classification tagged or otherwise identifiable,10: Enforced Policy with tagged/identifiable classifications"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H30">
-      <formula1>"0: 0%,1: 10%,2: 20%,3: 30%,4: 40%,5: 50%,6: 60%,7: 70%,8: 80%,9: 90%,10: Near 100%"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H31">
-      <formula1>"0: No items completed,5: 1 item completed,10: 2 items completed"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H32">
-      <formula1>"0: 0%,1: 10%,2: 20%,3: 30%,4: 40%,5: 50%,6: 60%,7: 70%,8: 80% ,9: 90%,10: Near 100%"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H33">
-      <formula1>"0: No items completed,5: 1 item  completed,10: 2 items completed"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H34">
-      <formula1>"0: 0%,1: 10%,2: 20%,3: 30%,4: 40%,5: 50%,6: 60%,7: 70%,8: 80%,9: 90%,10: Near 100%"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H35">
-      <formula1>"0: 0%,1: 10%,2: 20%,3: 30%,4: 40%,5: 50%,6: 60%,7: 70%,8: 80%,9: 90%,10: Near 100%"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H36">
-      <formula1>"0: No items completed,3: 1 item completed,5: 2 items completed,8: 3 items completed,10: 4 items completed"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H37">
-      <formula1>"0: No items completed,2: 1 item completed,4: 2 items completed,6: 3 items completed,8: 4 items completed,10: 5 items completed"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H38">
-      <formula1>"0: No items completed,2: 1 item completed,4: 2 items completed,5: 3 items completed,7: 4 items completed,9: 5 items completed,10: 6 items completed"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H39">
-      <formula1>"0: No alerting to any owners,1: Alerting in at least one owner,3: Alerting to some owners [&gt;20%],6: Alerting to most owners [&gt;60%],10: Alerting to all owners [100%]"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H40">
-      <formula1>"0: No items completed,2: 1 item completed,3: 2 items completed,4: 3 items completed,5: 4 items completed,7: 5 items completed,8: 6 items completed,9: 7 items completed,10: 8 items completed"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H41">
-      <formula1>"0: Never,1: Monthly or greater,2: More than a week,3: 7 days,4: 5 days,6: 2 days,8: 1 day,10: Instant"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H42">
-      <formula1>"0: No items completed,2: 1 items completed,3: 2 items completed,5: 3 items completed,6: 4 items completed,8: 5 items completed,9: 6 items completed,10: 7 items completed"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H43">
-      <formula1>"0: No items completed,2: 1 items completed,3: 2 items completed,5: 3 items completed,6: 4 items completed,8: 5 items completed,9: 6 items completed,10: 7 items completed"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H44">
-      <formula1>"0: Never,1: Monthly or greater,2: More than a week,3: 7 days,4: 5 days,6: 2 days,8: 1 day,10: Instant"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H45">
-      <formula1>"0: No items completed,3: 1 item completed,5: 2 items completed,8: 3 items completed,10: 4 items completed"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H46">
-      <formula1>"0: No items completed,3: 1 item completed,5: 2 items completed,8: 3 items completed,10: 4 items completed"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H47">
-      <formula1>"0: No alerting in workflow tools,1: Alerting in at least one tool,3: Alerting in some tooling [&gt;20%],6: Alerting in most tooling [&gt;60%],10: Alerting in all workflow tools [100%]"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H48">
-      <formula1>"0: No review of trends,3: Manual review of trends,6: Automated trend detection,10: Manual review and automated trend detection"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H49">
-      <formula1>"0: Does not exist,10: Exists"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H50">
-      <formula1>"0: Does not exist,10: Exists"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H51">
-      <formula1>"0: No items completed,3: 1 item completed,5: 2 items completed,8: 3 items completed,10: 4 items completed"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H52">
-      <formula1>"0: None,1: Annual,2: Quarterly,5: Monthly,7: Bi-Weekly,8: Weekly,10: Daily"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H53">
       <formula1>"0: 0%,1: 10%,2: 20%,3: 30%,4: 40%,5: 50%,6: 60%,7: 70%,8: 80%,9: 90%,10: Near 100%"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H54">
-      <formula1>"0: No alerting,10: Alerting exists"</formula1>
+      <formula1>"0: Not done,10: Completed"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H55">
-      <formula1>"0: No items completed,3: 1 item completed,5: 2 items completed,8: 3 items completed,10: 4 items completed"</formula1>
+      <formula1>"0: Not done,10: Completed"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H56">
-      <formula1>"0: No items completed,2: 1 item completed,4: 2 items completed,6: 3 items completed,8: 4 items completed,10: 5 items completed"</formula1>
+      <formula1>"0: Not done,10: Completed"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H57">
-      <formula1>"0: No items completed,2: 1 item completed,4: 2 items completed,6: 3 items completed,8: 4 items completed,10: 5 items completed"</formula1>
+      <formula1>"0: No items completed,5: 1 item completed,10: 2 items completed"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H58">
-      <formula1>"0: No items completed,2: 1 item completed,4: 2 items completed,6: 3 items completed,8: 4 items completed,10: 5 items completed"</formula1>
+      <formula1>"0: 0%,1: 10%,2: 20%,3: 30%,4: 40%,5: 50%,6: 60%,7: 70%,8: 80% ,9: 90%,10: Near 100%"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H59">
-      <formula1>"0: No items completed,5: item 1 completed,10: item 2 completed"</formula1>
+      <formula1>"0: No items completed,5: 1 item  completed,10: 2 items completed"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H60">
-      <formula1>"0: No items completed,4: 1 item completed,7: 2 items completed,10: 3 items completed"</formula1>
+      <formula1>"0: 0%,1: 10%,2: 20%,3: 30%,4: 40%,5: 50%,6: 60%,7: 70%,8: 80%,9: 90%,10: Near 100%"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H61">
       <formula1>"0: 0%,1: 10%,2: 20%,3: 30%,4: 40%,5: 50%,6: 60%,7: 70%,8: 80%,9: 90%,10: Near 100%"</formula1>
@@ -4709,24 +5904,126 @@
       <formula1>"0: No items completed,3: 1 item completed,5: 2 items completed,8: 3 items completed,10: 4 items completed"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H63">
-      <formula1>"0: No items completed,3: 1 item completed,5: 2 items completed,8: 3 items completed,10: 4 items completed"</formula1>
+      <formula1>"0: No items completed,2: 1 item completed,4: 2 items completed,6: 3 items completed,8: 4 items completed,10: 5 items completed"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H64">
       <formula1>"0: No items completed,2: 1 item completed,4: 2 items completed,5: 3 items completed,7: 4 items completed,9: 5 items completed,10: 6 items completed"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H65">
+      <formula1>"0: No alerting to any owners,1: Alerting in at least one owner,3: Alerting to some owners [&gt;20%],6: Alerting to most owners [&gt;60%],10: Alerting to all owners [100%]"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H66">
+      <formula1>"0: No items completed,2: 1 item completed,3: 2 items completed,4: 3 items completed,5: 4 items completed,7: 5 items completed,8: 6 items completed,9: 7 items completed,10: 8 items completed"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H67">
+      <formula1>"0: Never,1: Monthly or greater,2: More than a week,3: 7 days,4: 5 days,6: 2 days,8: 1 day,10: Instant"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H68">
+      <formula1>"0: No items completed,2: 1 items completed,3: 2 items completed,5: 3 items completed,6: 4 items completed,8: 5 items completed,9: 6 items completed,10: 7 items completed"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H69">
+      <formula1>"0: No items completed,2: 1 items completed,3: 2 items completed,5: 3 items completed,6: 4 items completed,8: 5 items completed,9: 6 items completed,10: 7 items completed"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H70">
+      <formula1>"0: Never,1: Monthly or greater,2: More than a week,3: 7 days,4: 5 days,6: 2 days,8: 1 day,10: Instant"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H71">
+      <formula1>"0: Not done,10: Completed"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H72">
+      <formula1>"0: No items completed,3: 1 item completed,5: 2 items completed,8: 3 items completed,10: 4 items completed"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H73">
+      <formula1>"0: No items completed,3: 1 item completed,5: 2 items completed,8: 3 items completed,10: 4 items completed"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H74">
+      <formula1>"0: Not done,10: Completed"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H75">
+      <formula1>"0: No alerting in workflow tools,1: Alerting in at least one tool,3: Alerting in some tooling [&gt;20%],6: Alerting in most tooling [&gt;60%],10: Alerting in all workflow tools [100%]"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H76">
+      <formula1>"0: Not done,10: Completed"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H77">
+      <formula1>"0: Not done,10: Completed"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H78">
+      <formula1>"0: No review of trends,3: Manual review of trends,6: Automated trend detection,10: Manual review and automated trend detection"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H79">
+      <formula1>"0: Does not exist,10: Exists"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H80">
+      <formula1>"0: Does not exist,10: Exists"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H81">
+      <formula1>"0: Not done,10: Completed"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H82">
+      <formula1>"0: Not done,10: Completed"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H83">
+      <formula1>"0: Not done,10: Completed"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H84">
+      <formula1>"0: Not done,10: Completed"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H85">
+      <formula1>"0: No items completed,3: 1 item completed,5: 2 items completed,8: 3 items completed,10: 4 items completed"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H86">
+      <formula1>"0: None,1: Annual,2: Quarterly,5: Monthly,7: Bi-Weekly,8: Weekly,10: Daily"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H87">
+      <formula1>"0: 0%,1: 10%,2: 20%,3: 30%,4: 40%,5: 50%,6: 60%,7: 70%,8: 80%,9: 90%,10: Near 100%"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H88">
+      <formula1>"0: No alerting,10: Alerting exists"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H89">
+      <formula1>"0: No items completed,3: 1 item completed,5: 2 items completed,8: 3 items completed,10: 4 items completed"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H90">
+      <formula1>"0: No items completed,2: 1 item completed,4: 2 items completed,6: 3 items completed,8: 4 items completed,10: 5 items completed"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H91">
+      <formula1>"0: No items completed,2: 1 item completed,4: 2 items completed,6: 3 items completed,8: 4 items completed,10: 5 items completed"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H92">
+      <formula1>"0: No items completed,2: 1 item completed,4: 2 items completed,6: 3 items completed,8: 4 items completed,10: 5 items completed"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H93">
+      <formula1>"0: No items completed,5: item 1 completed,10: item 2 completed"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H94">
+      <formula1>"0: No items completed,4: 1 item completed,7: 2 items completed,10: 3 items completed"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H95">
+      <formula1>"0: 0%,1: 10%,2: 20%,3: 30%,4: 40%,5: 50%,6: 60%,7: 70%,8: 80%,9: 90%,10: Near 100%"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H96">
+      <formula1>"0: No items completed,3: 1 item completed,5: 2 items completed,8: 3 items completed,10: 4 items completed"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H97">
+      <formula1>"0: No items completed,3: 1 item completed,5: 2 items completed,8: 3 items completed,10: 4 items completed"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H98">
       <formula1>"0: No items completed,2: 1 item completed,4: 2 items completed,5: 3 items completed,7: 4 items completed,9: 5 items completed,10: 6 items completed"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H66">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H99">
+      <formula1>"0: No items completed,2: 1 item completed,4: 2 items completed,5: 3 items completed,7: 4 items completed,9: 5 items completed,10: 6 items completed"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H100">
       <formula1>"0: No items completed,3: 1 item completed,5: 2 items completed,8: 3 items completed,10: 4 items completed"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H67">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H101">
       <formula1>"0: No items completed,3: 1 item completed,5: 2 items completed,8: 3 items completed,10: 4 items completed"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H68">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H102">
       <formula1>"0: None,10: communicates wins in KPI thresholds and unit costs"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H69">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H103">
       <formula1>"0: Not monitored,2: Reported,5: Manual remediation,10: Automated remediation"</formula1>
     </dataValidation>
   </dataValidations>
@@ -4799,6 +6096,40 @@
     <hyperlink ref="D67" r:id="rId66"/>
     <hyperlink ref="D68" r:id="rId67"/>
     <hyperlink ref="D69" r:id="rId68"/>
+    <hyperlink ref="D70" r:id="rId69"/>
+    <hyperlink ref="D71" r:id="rId70"/>
+    <hyperlink ref="D72" r:id="rId71"/>
+    <hyperlink ref="D73" r:id="rId72"/>
+    <hyperlink ref="D74" r:id="rId73"/>
+    <hyperlink ref="D75" r:id="rId74"/>
+    <hyperlink ref="D76" r:id="rId75"/>
+    <hyperlink ref="D77" r:id="rId76"/>
+    <hyperlink ref="D78" r:id="rId77"/>
+    <hyperlink ref="D79" r:id="rId78"/>
+    <hyperlink ref="D80" r:id="rId79"/>
+    <hyperlink ref="D81" r:id="rId80"/>
+    <hyperlink ref="D82" r:id="rId81"/>
+    <hyperlink ref="D83" r:id="rId82"/>
+    <hyperlink ref="D84" r:id="rId83"/>
+    <hyperlink ref="D85" r:id="rId84"/>
+    <hyperlink ref="D86" r:id="rId85"/>
+    <hyperlink ref="D87" r:id="rId86"/>
+    <hyperlink ref="D88" r:id="rId87"/>
+    <hyperlink ref="D89" r:id="rId88"/>
+    <hyperlink ref="D90" r:id="rId89"/>
+    <hyperlink ref="D91" r:id="rId90"/>
+    <hyperlink ref="D92" r:id="rId91"/>
+    <hyperlink ref="D93" r:id="rId92"/>
+    <hyperlink ref="D94" r:id="rId93"/>
+    <hyperlink ref="D95" r:id="rId94"/>
+    <hyperlink ref="D96" r:id="rId95"/>
+    <hyperlink ref="D97" r:id="rId96"/>
+    <hyperlink ref="D98" r:id="rId97"/>
+    <hyperlink ref="D99" r:id="rId98"/>
+    <hyperlink ref="D100" r:id="rId99"/>
+    <hyperlink ref="D101" r:id="rId100"/>
+    <hyperlink ref="D102" r:id="rId101"/>
+    <hyperlink ref="D103" r:id="rId102"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>

</xml_diff>

<commit_message>
Enable generation to take variables
will allow overrides as needed
</commit_message>
<xml_diff>
--- a/assessments/FinOps++/assessment.xlsx
+++ b/assessments/FinOps++/assessment.xlsx
@@ -2935,7 +2935,7 @@
         <v>310</v>
       </c>
       <c r="F6">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="G6" s="1" t="s">
         <v>318</v>
@@ -3056,7 +3056,7 @@
         <v>311</v>
       </c>
       <c r="F10">
-        <v>1</v>
+        <v>100</v>
       </c>
       <c r="G10" s="1" t="s">
         <v>319</v>
@@ -3235,7 +3235,7 @@
         <v>310</v>
       </c>
       <c r="F16">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H16" s="1" t="s">
         <v>398</v>
@@ -3359,7 +3359,7 @@
         <v>309</v>
       </c>
       <c r="F20">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G20" s="1" t="s">
         <v>322</v>
@@ -3550,7 +3550,7 @@
         <v>309</v>
       </c>
       <c r="F26">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G26" s="1" t="s">
         <v>327</v>

</xml_diff>

<commit_message>
Fix off weight override feature
to include the variable suffix to let folks know it is an override
</commit_message>
<xml_diff>
--- a/assessments/FinOps++/assessment.xlsx
+++ b/assessments/FinOps++/assessment.xlsx
@@ -2935,7 +2935,7 @@
         <v>310</v>
       </c>
       <c r="F6">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="G6" s="1" t="s">
         <v>318</v>
@@ -3056,7 +3056,7 @@
         <v>311</v>
       </c>
       <c r="F10">
-        <v>100</v>
+        <v>1</v>
       </c>
       <c r="G10" s="1" t="s">
         <v>319</v>
@@ -3235,7 +3235,7 @@
         <v>310</v>
       </c>
       <c r="F16">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H16" s="1" t="s">
         <v>398</v>
@@ -3359,7 +3359,7 @@
         <v>309</v>
       </c>
       <c r="F20">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G20" s="1" t="s">
         <v>322</v>
@@ -3550,7 +3550,7 @@
         <v>309</v>
       </c>
       <c r="F26">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G26" s="1" t="s">
         <v>327</v>

</xml_diff>

<commit_message>
Fix linting and errors
</commit_message>
<xml_diff>
--- a/assessments/FinOps++/assessment.xlsx
+++ b/assessments/FinOps++/assessment.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1182" uniqueCount="414">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1184" uniqueCount="417">
   <si>
     <t>Sum of Weights</t>
   </si>
@@ -956,6 +956,9 @@
   </si>
   <si>
     <t>2.1.0</t>
+  </si>
+  <si>
+    <t>2.0.0</t>
   </si>
   <si>
     <t>1.6.1</t>
@@ -1118,6 +1121,21 @@
 * Define thresholds to change
 * Combine with architecture analysis for SP &amp; RIs
 10*Ceil(x/5)</t>
+  </si>
+  <si>
+    <t>* Implement architecture changes in time boxed iterations rather than big migrations
+* Track actual cost outcomes vs estimated savings documented in prior trade off analysis
+* Define and monitor success metrics (cost delta, performance, reliability) for each iteration
+* Hold structured retrospectives after each iteration to capture lessons learned
+* Feed iteration outcomes back into the modernization backlog to reprioritize remaining work
+10*Ceil(x/5)</t>
+  </si>
+  <si>
+    <t>* Document and publish cost savings and performance outcomes achieved through architecture changes
+* Update internal architecture reference guides and design patterns with validated approaches
+* Share case studies and reusable blueprints with engineering teams to accelerate adoption
+* Establish a regular cadence to refresh published benefits data and retire outdated references
+10*Ceil(x/4)</t>
   </si>
   <si>
     <t>* Process defined for new accounts and resources deployed
@@ -2810,10 +2828,10 @@
         <v>1</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>396</v>
+        <v>399</v>
       </c>
       <c r="I2">
         <f>F2*VALUE(LEFT(H2, FIND(":", H2)-1))</f>
@@ -2842,10 +2860,10 @@
         <v>1</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>397</v>
+        <v>400</v>
       </c>
       <c r="I3">
         <f>F3*VALUE(LEFT(H3, FIND(":", H3)-1))</f>
@@ -2874,10 +2892,10 @@
         <v>1</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="H4" s="1" t="s">
-        <v>397</v>
+        <v>400</v>
       </c>
       <c r="I4">
         <f>F4*VALUE(LEFT(H4, FIND(":", H4)-1))</f>
@@ -2906,10 +2924,10 @@
         <v>1</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>397</v>
+        <v>400</v>
       </c>
       <c r="I5">
         <f>F5*VALUE(LEFT(H5, FIND(":", H5)-1))</f>
@@ -2938,10 +2956,10 @@
         <v>1</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="H6" s="1" t="s">
-        <v>397</v>
+        <v>400</v>
       </c>
       <c r="I6">
         <f>F6*VALUE(LEFT(H6, FIND(":", H6)-1))</f>
@@ -2972,7 +2990,7 @@
         <v>1</v>
       </c>
       <c r="H7" s="1" t="s">
-        <v>398</v>
+        <v>401</v>
       </c>
       <c r="I7">
         <f>F7*VALUE(LEFT(H7, FIND(":", H7)-1))</f>
@@ -3001,7 +3019,7 @@
         <v>1</v>
       </c>
       <c r="H8" s="1" t="s">
-        <v>398</v>
+        <v>401</v>
       </c>
       <c r="I8">
         <f>F8*VALUE(LEFT(H8, FIND(":", H8)-1))</f>
@@ -3030,7 +3048,7 @@
         <v>1</v>
       </c>
       <c r="H9" s="1" t="s">
-        <v>398</v>
+        <v>401</v>
       </c>
       <c r="I9">
         <f>F9*VALUE(LEFT(H9, FIND(":", H9)-1))</f>
@@ -3059,10 +3077,10 @@
         <v>1</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="H10" s="1" t="s">
-        <v>397</v>
+        <v>400</v>
       </c>
       <c r="I10">
         <f>F10*VALUE(LEFT(H10, FIND(":", H10)-1))</f>
@@ -3091,7 +3109,7 @@
         <v>1</v>
       </c>
       <c r="H11" s="1" t="s">
-        <v>398</v>
+        <v>401</v>
       </c>
       <c r="I11">
         <f>F11*VALUE(LEFT(H11, FIND(":", H11)-1))</f>
@@ -3122,7 +3140,7 @@
         <v>1</v>
       </c>
       <c r="H12" s="1" t="s">
-        <v>398</v>
+        <v>401</v>
       </c>
       <c r="I12">
         <f>F12*VALUE(LEFT(H12, FIND(":", H12)-1))</f>
@@ -3151,7 +3169,7 @@
         <v>1</v>
       </c>
       <c r="H13" s="1" t="s">
-        <v>398</v>
+        <v>401</v>
       </c>
       <c r="I13">
         <f>F13*VALUE(LEFT(H13, FIND(":", H13)-1))</f>
@@ -3180,7 +3198,7 @@
         <v>1</v>
       </c>
       <c r="H14" s="1" t="s">
-        <v>398</v>
+        <v>401</v>
       </c>
       <c r="I14">
         <f>F14*VALUE(LEFT(H14, FIND(":", H14)-1))</f>
@@ -3209,7 +3227,7 @@
         <v>1</v>
       </c>
       <c r="H15" s="1" t="s">
-        <v>398</v>
+        <v>401</v>
       </c>
       <c r="I15">
         <f>F15*VALUE(LEFT(H15, FIND(":", H15)-1))</f>
@@ -3238,7 +3256,7 @@
         <v>1</v>
       </c>
       <c r="H16" s="1" t="s">
-        <v>398</v>
+        <v>401</v>
       </c>
       <c r="I16">
         <f>F16*VALUE(LEFT(H16, FIND(":", H16)-1))</f>
@@ -3267,7 +3285,7 @@
         <v>1</v>
       </c>
       <c r="H17" s="1" t="s">
-        <v>398</v>
+        <v>401</v>
       </c>
       <c r="I17">
         <f>F17*VALUE(LEFT(H17, FIND(":", H17)-1))</f>
@@ -3298,10 +3316,10 @@
         <v>1</v>
       </c>
       <c r="G18" s="1" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="H18" s="1" t="s">
-        <v>399</v>
+        <v>402</v>
       </c>
       <c r="I18">
         <f>F18*VALUE(LEFT(H18, FIND(":", H18)-1))</f>
@@ -3330,10 +3348,10 @@
         <v>1</v>
       </c>
       <c r="G19" s="1" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="H19" s="1" t="s">
-        <v>400</v>
+        <v>403</v>
       </c>
       <c r="I19">
         <f>F19*VALUE(LEFT(H19, FIND(":", H19)-1))</f>
@@ -3362,10 +3380,10 @@
         <v>1</v>
       </c>
       <c r="G20" s="1" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="H20" s="1" t="s">
-        <v>401</v>
+        <v>404</v>
       </c>
       <c r="I20">
         <f>F20*VALUE(LEFT(H20, FIND(":", H20)-1))</f>
@@ -3394,10 +3412,10 @@
         <v>1</v>
       </c>
       <c r="G21" s="1" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="H21" s="1" t="s">
-        <v>397</v>
+        <v>400</v>
       </c>
       <c r="I21">
         <f>F21*VALUE(LEFT(H21, FIND(":", H21)-1))</f>
@@ -3426,7 +3444,7 @@
         <v>1</v>
       </c>
       <c r="H22" s="1" t="s">
-        <v>398</v>
+        <v>401</v>
       </c>
       <c r="I22">
         <f>F22*VALUE(LEFT(H22, FIND(":", H22)-1))</f>
@@ -3457,10 +3475,10 @@
         <v>1</v>
       </c>
       <c r="G23" s="1" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="H23" s="1" t="s">
-        <v>397</v>
+        <v>400</v>
       </c>
       <c r="I23">
         <f>F23*VALUE(LEFT(H23, FIND(":", H23)-1))</f>
@@ -3489,10 +3507,10 @@
         <v>1</v>
       </c>
       <c r="G24" s="1" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="H24" s="1" t="s">
-        <v>397</v>
+        <v>400</v>
       </c>
       <c r="I24">
         <f>F24*VALUE(LEFT(H24, FIND(":", H24)-1))</f>
@@ -3521,10 +3539,10 @@
         <v>1</v>
       </c>
       <c r="G25" s="1" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="H25" s="1" t="s">
-        <v>397</v>
+        <v>400</v>
       </c>
       <c r="I25">
         <f>F25*VALUE(LEFT(H25, FIND(":", H25)-1))</f>
@@ -3553,10 +3571,10 @@
         <v>1</v>
       </c>
       <c r="G26" s="1" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="H26" s="1" t="s">
-        <v>397</v>
+        <v>400</v>
       </c>
       <c r="I26">
         <f>F26*VALUE(LEFT(H26, FIND(":", H26)-1))</f>
@@ -3585,10 +3603,10 @@
         <v>1</v>
       </c>
       <c r="G27" s="1" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="H27" s="1" t="s">
-        <v>397</v>
+        <v>400</v>
       </c>
       <c r="I27">
         <f>F27*VALUE(LEFT(H27, FIND(":", H27)-1))</f>
@@ -3617,10 +3635,10 @@
         <v>1</v>
       </c>
       <c r="G28" s="1" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="H28" s="1" t="s">
-        <v>397</v>
+        <v>400</v>
       </c>
       <c r="I28">
         <f>F28*VALUE(LEFT(H28, FIND(":", H28)-1))</f>
@@ -3651,7 +3669,7 @@
         <v>1</v>
       </c>
       <c r="H29" s="1" t="s">
-        <v>398</v>
+        <v>401</v>
       </c>
       <c r="I29">
         <f>F29*VALUE(LEFT(H29, FIND(":", H29)-1))</f>
@@ -3680,7 +3698,7 @@
         <v>1</v>
       </c>
       <c r="H30" s="1" t="s">
-        <v>398</v>
+        <v>401</v>
       </c>
       <c r="I30">
         <f>F30*VALUE(LEFT(H30, FIND(":", H30)-1))</f>
@@ -3709,7 +3727,7 @@
         <v>1</v>
       </c>
       <c r="H31" s="1" t="s">
-        <v>398</v>
+        <v>401</v>
       </c>
       <c r="I31">
         <f>F31*VALUE(LEFT(H31, FIND(":", H31)-1))</f>
@@ -3738,7 +3756,7 @@
         <v>1</v>
       </c>
       <c r="H32" s="1" t="s">
-        <v>398</v>
+        <v>401</v>
       </c>
       <c r="I32">
         <f>F32*VALUE(LEFT(H32, FIND(":", H32)-1))</f>
@@ -3767,7 +3785,7 @@
         <v>1</v>
       </c>
       <c r="H33" s="1" t="s">
-        <v>398</v>
+        <v>401</v>
       </c>
       <c r="I33">
         <f>F33*VALUE(LEFT(H33, FIND(":", H33)-1))</f>
@@ -3796,7 +3814,7 @@
         <v>1</v>
       </c>
       <c r="H34" s="1" t="s">
-        <v>398</v>
+        <v>401</v>
       </c>
       <c r="I34">
         <f>F34*VALUE(LEFT(H34, FIND(":", H34)-1))</f>
@@ -3827,7 +3845,7 @@
         <v>1</v>
       </c>
       <c r="H35" s="1" t="s">
-        <v>402</v>
+        <v>405</v>
       </c>
       <c r="I35">
         <f>F35*VALUE(LEFT(H35, FIND(":", H35)-1))</f>
@@ -3856,10 +3874,10 @@
         <v>1</v>
       </c>
       <c r="G36" s="1" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="H36" s="1" t="s">
-        <v>397</v>
+        <v>400</v>
       </c>
       <c r="I36">
         <f>F36*VALUE(LEFT(H36, FIND(":", H36)-1))</f>
@@ -3888,10 +3906,10 @@
         <v>1</v>
       </c>
       <c r="G37" s="1" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="H37" s="1" t="s">
-        <v>397</v>
+        <v>400</v>
       </c>
       <c r="I37">
         <f>F37*VALUE(LEFT(H37, FIND(":", H37)-1))</f>
@@ -3920,10 +3938,10 @@
         <v>1</v>
       </c>
       <c r="G38" s="1" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="H38" s="1" t="s">
-        <v>397</v>
+        <v>400</v>
       </c>
       <c r="I38">
         <f>F38*VALUE(LEFT(H38, FIND(":", H38)-1))</f>
@@ -3956,7 +3974,7 @@
         <v>1</v>
       </c>
       <c r="H39" s="1" t="s">
-        <v>403</v>
+        <v>406</v>
       </c>
       <c r="I39">
         <f>F39*VALUE(LEFT(H39, FIND(":", H39)-1))</f>
@@ -3985,10 +4003,10 @@
         <v>1</v>
       </c>
       <c r="G40" s="1" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="H40" s="1" t="s">
-        <v>397</v>
+        <v>400</v>
       </c>
       <c r="I40">
         <f>F40*VALUE(LEFT(H40, FIND(":", H40)-1))</f>
@@ -4017,7 +4035,7 @@
         <v>1</v>
       </c>
       <c r="H41" s="1" t="s">
-        <v>404</v>
+        <v>407</v>
       </c>
       <c r="I41">
         <f>F41*VALUE(LEFT(H41, FIND(":", H41)-1))</f>
@@ -4040,13 +4058,16 @@
         <v>216</v>
       </c>
       <c r="E42" t="s">
-        <v>310</v>
+        <v>313</v>
       </c>
       <c r="F42">
         <v>1</v>
       </c>
+      <c r="G42" s="1" t="s">
+        <v>335</v>
+      </c>
       <c r="H42" s="1" t="s">
-        <v>398</v>
+        <v>400</v>
       </c>
       <c r="I42">
         <f>F42*VALUE(LEFT(H42, FIND(":", H42)-1))</f>
@@ -4069,13 +4090,16 @@
         <v>217</v>
       </c>
       <c r="E43" t="s">
-        <v>310</v>
+        <v>313</v>
       </c>
       <c r="F43">
         <v>1</v>
       </c>
+      <c r="G43" s="1" t="s">
+        <v>336</v>
+      </c>
       <c r="H43" s="1" t="s">
-        <v>398</v>
+        <v>400</v>
       </c>
       <c r="I43">
         <f>F43*VALUE(LEFT(H43, FIND(":", H43)-1))</f>
@@ -4104,7 +4128,7 @@
         <v>1</v>
       </c>
       <c r="H44" s="1" t="s">
-        <v>398</v>
+        <v>401</v>
       </c>
       <c r="I44">
         <f>F44*VALUE(LEFT(H44, FIND(":", H44)-1))</f>
@@ -4133,7 +4157,7 @@
         <v>1</v>
       </c>
       <c r="H45" s="1" t="s">
-        <v>398</v>
+        <v>401</v>
       </c>
       <c r="I45">
         <f>F45*VALUE(LEFT(H45, FIND(":", H45)-1))</f>
@@ -4162,7 +4186,7 @@
         <v>1</v>
       </c>
       <c r="H46" s="1" t="s">
-        <v>398</v>
+        <v>401</v>
       </c>
       <c r="I46">
         <f>F46*VALUE(LEFT(H46, FIND(":", H46)-1))</f>
@@ -4191,10 +4215,10 @@
         <v>1</v>
       </c>
       <c r="G47" s="1" t="s">
-        <v>334</v>
+        <v>337</v>
       </c>
       <c r="H47" s="1" t="s">
-        <v>397</v>
+        <v>400</v>
       </c>
       <c r="I47">
         <f>F47*VALUE(LEFT(H47, FIND(":", H47)-1))</f>
@@ -4223,7 +4247,7 @@
         <v>1</v>
       </c>
       <c r="H48" s="1" t="s">
-        <v>398</v>
+        <v>401</v>
       </c>
       <c r="I48">
         <f>F48*VALUE(LEFT(H48, FIND(":", H48)-1))</f>
@@ -4252,7 +4276,7 @@
         <v>1</v>
       </c>
       <c r="H49" s="1" t="s">
-        <v>398</v>
+        <v>401</v>
       </c>
       <c r="I49">
         <f>F49*VALUE(LEFT(H49, FIND(":", H49)-1))</f>
@@ -4281,7 +4305,7 @@
         <v>1</v>
       </c>
       <c r="H50" s="1" t="s">
-        <v>398</v>
+        <v>401</v>
       </c>
       <c r="I50">
         <f>F50*VALUE(LEFT(H50, FIND(":", H50)-1))</f>
@@ -4312,7 +4336,7 @@
         <v>1</v>
       </c>
       <c r="H51" s="1" t="s">
-        <v>405</v>
+        <v>408</v>
       </c>
       <c r="I51">
         <f>F51*VALUE(LEFT(H51, FIND(":", H51)-1))</f>
@@ -4341,7 +4365,7 @@
         <v>1</v>
       </c>
       <c r="H52" s="1" t="s">
-        <v>398</v>
+        <v>401</v>
       </c>
       <c r="I52">
         <f>F52*VALUE(LEFT(H52, FIND(":", H52)-1))</f>
@@ -4370,7 +4394,7 @@
         <v>1</v>
       </c>
       <c r="H53" s="1" t="s">
-        <v>398</v>
+        <v>401</v>
       </c>
       <c r="I53">
         <f>F53*VALUE(LEFT(H53, FIND(":", H53)-1))</f>
@@ -4399,7 +4423,7 @@
         <v>1</v>
       </c>
       <c r="H54" s="1" t="s">
-        <v>398</v>
+        <v>401</v>
       </c>
       <c r="I54">
         <f>F54*VALUE(LEFT(H54, FIND(":", H54)-1))</f>
@@ -4428,7 +4452,7 @@
         <v>1</v>
       </c>
       <c r="H55" s="1" t="s">
-        <v>398</v>
+        <v>401</v>
       </c>
       <c r="I55">
         <f>F55*VALUE(LEFT(H55, FIND(":", H55)-1))</f>
@@ -4457,7 +4481,7 @@
         <v>1</v>
       </c>
       <c r="H56" s="1" t="s">
-        <v>398</v>
+        <v>401</v>
       </c>
       <c r="I56">
         <f>F56*VALUE(LEFT(H56, FIND(":", H56)-1))</f>
@@ -4488,7 +4512,7 @@
         <v>1</v>
       </c>
       <c r="H57" s="1" t="s">
-        <v>398</v>
+        <v>401</v>
       </c>
       <c r="I57">
         <f>F57*VALUE(LEFT(H57, FIND(":", H57)-1))</f>
@@ -4517,7 +4541,7 @@
         <v>1</v>
       </c>
       <c r="H58" s="1" t="s">
-        <v>398</v>
+        <v>401</v>
       </c>
       <c r="I58">
         <f>F58*VALUE(LEFT(H58, FIND(":", H58)-1))</f>
@@ -4546,7 +4570,7 @@
         <v>1</v>
       </c>
       <c r="H59" s="1" t="s">
-        <v>398</v>
+        <v>401</v>
       </c>
       <c r="I59">
         <f>F59*VALUE(LEFT(H59, FIND(":", H59)-1))</f>
@@ -4575,7 +4599,7 @@
         <v>1</v>
       </c>
       <c r="H60" s="1" t="s">
-        <v>398</v>
+        <v>401</v>
       </c>
       <c r="I60">
         <f>F60*VALUE(LEFT(H60, FIND(":", H60)-1))</f>
@@ -4604,7 +4628,7 @@
         <v>1</v>
       </c>
       <c r="H61" s="1" t="s">
-        <v>398</v>
+        <v>401</v>
       </c>
       <c r="I61">
         <f>F61*VALUE(LEFT(H61, FIND(":", H61)-1))</f>
@@ -4633,10 +4657,10 @@
         <v>1</v>
       </c>
       <c r="G62" s="1" t="s">
-        <v>335</v>
+        <v>338</v>
       </c>
       <c r="H62" s="1" t="s">
-        <v>397</v>
+        <v>400</v>
       </c>
       <c r="I62">
         <f>F62*VALUE(LEFT(H62, FIND(":", H62)-1))</f>
@@ -4667,7 +4691,7 @@
         <v>1</v>
       </c>
       <c r="H63" s="1" t="s">
-        <v>398</v>
+        <v>401</v>
       </c>
       <c r="I63">
         <f>F63*VALUE(LEFT(H63, FIND(":", H63)-1))</f>
@@ -4696,7 +4720,7 @@
         <v>1</v>
       </c>
       <c r="H64" s="1" t="s">
-        <v>406</v>
+        <v>409</v>
       </c>
       <c r="I64">
         <f>F64*VALUE(LEFT(H64, FIND(":", H64)-1))</f>
@@ -4725,7 +4749,7 @@
         <v>1</v>
       </c>
       <c r="H65" s="1" t="s">
-        <v>405</v>
+        <v>408</v>
       </c>
       <c r="I65">
         <f>F65*VALUE(LEFT(H65, FIND(":", H65)-1))</f>
@@ -4754,7 +4778,7 @@
         <v>1</v>
       </c>
       <c r="H66" s="1" t="s">
-        <v>398</v>
+        <v>401</v>
       </c>
       <c r="I66">
         <f>F66*VALUE(LEFT(H66, FIND(":", H66)-1))</f>
@@ -4783,7 +4807,7 @@
         <v>1</v>
       </c>
       <c r="H67" s="1" t="s">
-        <v>398</v>
+        <v>401</v>
       </c>
       <c r="I67">
         <f>F67*VALUE(LEFT(H67, FIND(":", H67)-1))</f>
@@ -4812,7 +4836,7 @@
         <v>1</v>
       </c>
       <c r="H68" s="1" t="s">
-        <v>398</v>
+        <v>401</v>
       </c>
       <c r="I68">
         <f>F68*VALUE(LEFT(H68, FIND(":", H68)-1))</f>
@@ -4843,10 +4867,10 @@
         <v>1</v>
       </c>
       <c r="G69" s="1" t="s">
-        <v>336</v>
+        <v>339</v>
       </c>
       <c r="H69" s="1" t="s">
-        <v>397</v>
+        <v>400</v>
       </c>
       <c r="I69">
         <f>F69*VALUE(LEFT(H69, FIND(":", H69)-1))</f>
@@ -4875,10 +4899,10 @@
         <v>1</v>
       </c>
       <c r="G70" s="1" t="s">
-        <v>337</v>
+        <v>340</v>
       </c>
       <c r="H70" s="1" t="s">
-        <v>405</v>
+        <v>408</v>
       </c>
       <c r="I70">
         <f>F70*VALUE(LEFT(H70, FIND(":", H70)-1))</f>
@@ -4907,10 +4931,10 @@
         <v>1</v>
       </c>
       <c r="G71" s="1" t="s">
-        <v>338</v>
+        <v>341</v>
       </c>
       <c r="H71" s="1" t="s">
-        <v>397</v>
+        <v>400</v>
       </c>
       <c r="I71">
         <f>F71*VALUE(LEFT(H71, FIND(":", H71)-1))</f>
@@ -4939,10 +4963,10 @@
         <v>1</v>
       </c>
       <c r="G72" s="1" t="s">
-        <v>339</v>
+        <v>342</v>
       </c>
       <c r="H72" s="1" t="s">
-        <v>405</v>
+        <v>408</v>
       </c>
       <c r="I72">
         <f>F72*VALUE(LEFT(H72, FIND(":", H72)-1))</f>
@@ -4971,10 +4995,10 @@
         <v>1</v>
       </c>
       <c r="G73" s="1" t="s">
-        <v>340</v>
+        <v>343</v>
       </c>
       <c r="H73" s="1" t="s">
-        <v>405</v>
+        <v>408</v>
       </c>
       <c r="I73">
         <f>F73*VALUE(LEFT(H73, FIND(":", H73)-1))</f>
@@ -5003,10 +5027,10 @@
         <v>1</v>
       </c>
       <c r="G74" s="1" t="s">
-        <v>341</v>
+        <v>344</v>
       </c>
       <c r="H74" s="1" t="s">
-        <v>397</v>
+        <v>400</v>
       </c>
       <c r="I74">
         <f>F74*VALUE(LEFT(H74, FIND(":", H74)-1))</f>
@@ -5035,7 +5059,7 @@
         <v>1</v>
       </c>
       <c r="H75" s="1" t="s">
-        <v>398</v>
+        <v>401</v>
       </c>
       <c r="I75">
         <f>F75*VALUE(LEFT(H75, FIND(":", H75)-1))</f>
@@ -5066,10 +5090,10 @@
         <v>1</v>
       </c>
       <c r="G76" s="1" t="s">
-        <v>342</v>
+        <v>345</v>
       </c>
       <c r="H76" s="1" t="s">
-        <v>397</v>
+        <v>400</v>
       </c>
       <c r="I76">
         <f>F76*VALUE(LEFT(H76, FIND(":", H76)-1))</f>
@@ -5098,10 +5122,10 @@
         <v>1</v>
       </c>
       <c r="G77" s="1" t="s">
-        <v>343</v>
+        <v>346</v>
       </c>
       <c r="H77" s="1" t="s">
-        <v>397</v>
+        <v>400</v>
       </c>
       <c r="I77">
         <f>F77*VALUE(LEFT(H77, FIND(":", H77)-1))</f>
@@ -5130,7 +5154,7 @@
         <v>1</v>
       </c>
       <c r="H78" s="1" t="s">
-        <v>407</v>
+        <v>410</v>
       </c>
       <c r="I78">
         <f>F78*VALUE(LEFT(H78, FIND(":", H78)-1))</f>
@@ -5159,7 +5183,7 @@
         <v>1</v>
       </c>
       <c r="H79" s="1" t="s">
-        <v>398</v>
+        <v>401</v>
       </c>
       <c r="I79">
         <f>F79*VALUE(LEFT(H79, FIND(":", H79)-1))</f>
@@ -5188,7 +5212,7 @@
         <v>1</v>
       </c>
       <c r="H80" s="1" t="s">
-        <v>398</v>
+        <v>401</v>
       </c>
       <c r="I80">
         <f>F80*VALUE(LEFT(H80, FIND(":", H80)-1))</f>
@@ -5217,10 +5241,10 @@
         <v>1</v>
       </c>
       <c r="G81" s="1" t="s">
-        <v>344</v>
+        <v>347</v>
       </c>
       <c r="H81" s="1" t="s">
-        <v>397</v>
+        <v>400</v>
       </c>
       <c r="I81">
         <f>F81*VALUE(LEFT(H81, FIND(":", H81)-1))</f>
@@ -5249,7 +5273,7 @@
         <v>1</v>
       </c>
       <c r="H82" s="1" t="s">
-        <v>398</v>
+        <v>401</v>
       </c>
       <c r="I82">
         <f>F82*VALUE(LEFT(H82, FIND(":", H82)-1))</f>
@@ -5280,7 +5304,7 @@
         <v>1</v>
       </c>
       <c r="H83" s="1" t="s">
-        <v>398</v>
+        <v>401</v>
       </c>
       <c r="I83">
         <f>F83*VALUE(LEFT(H83, FIND(":", H83)-1))</f>
@@ -5309,7 +5333,7 @@
         <v>1</v>
       </c>
       <c r="H84" s="1" t="s">
-        <v>398</v>
+        <v>401</v>
       </c>
       <c r="I84">
         <f>F84*VALUE(LEFT(H84, FIND(":", H84)-1))</f>
@@ -5338,7 +5362,7 @@
         <v>1</v>
       </c>
       <c r="H85" s="1" t="s">
-        <v>398</v>
+        <v>401</v>
       </c>
       <c r="I85">
         <f>F85*VALUE(LEFT(H85, FIND(":", H85)-1))</f>
@@ -5367,7 +5391,7 @@
         <v>1</v>
       </c>
       <c r="H86" s="1" t="s">
-        <v>408</v>
+        <v>411</v>
       </c>
       <c r="I86">
         <f>F86*VALUE(LEFT(H86, FIND(":", H86)-1))</f>
@@ -5396,7 +5420,7 @@
         <v>1</v>
       </c>
       <c r="H87" s="1" t="s">
-        <v>398</v>
+        <v>401</v>
       </c>
       <c r="I87">
         <f>F87*VALUE(LEFT(H87, FIND(":", H87)-1))</f>
@@ -5425,10 +5449,10 @@
         <v>1</v>
       </c>
       <c r="G88" s="1" t="s">
-        <v>345</v>
+        <v>348</v>
       </c>
       <c r="H88" s="1" t="s">
-        <v>397</v>
+        <v>400</v>
       </c>
       <c r="I88">
         <f>F88*VALUE(LEFT(H88, FIND(":", H88)-1))</f>
@@ -5457,10 +5481,10 @@
         <v>1</v>
       </c>
       <c r="G89" s="1" t="s">
-        <v>346</v>
+        <v>349</v>
       </c>
       <c r="H89" s="1" t="s">
-        <v>397</v>
+        <v>400</v>
       </c>
       <c r="I89">
         <f>F89*VALUE(LEFT(H89, FIND(":", H89)-1))</f>
@@ -5489,7 +5513,7 @@
         <v>1</v>
       </c>
       <c r="H90" s="1" t="s">
-        <v>398</v>
+        <v>401</v>
       </c>
       <c r="I90">
         <f>F90*VALUE(LEFT(H90, FIND(":", H90)-1))</f>
@@ -5512,13 +5536,13 @@
         <v>265</v>
       </c>
       <c r="E91" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="F91">
         <v>1</v>
       </c>
       <c r="H91" s="1" t="s">
-        <v>408</v>
+        <v>411</v>
       </c>
       <c r="I91">
         <f>F91*VALUE(LEFT(H91, FIND(":", H91)-1))</f>
@@ -5549,7 +5573,7 @@
         <v>1</v>
       </c>
       <c r="H92" s="1" t="s">
-        <v>398</v>
+        <v>401</v>
       </c>
       <c r="I92">
         <f>F92*VALUE(LEFT(H92, FIND(":", H92)-1))</f>
@@ -5578,10 +5602,10 @@
         <v>1</v>
       </c>
       <c r="G93" s="1" t="s">
-        <v>347</v>
+        <v>350</v>
       </c>
       <c r="H93" s="1" t="s">
-        <v>397</v>
+        <v>400</v>
       </c>
       <c r="I93">
         <f>F93*VALUE(LEFT(H93, FIND(":", H93)-1))</f>
@@ -5610,10 +5634,10 @@
         <v>1</v>
       </c>
       <c r="G94" s="1" t="s">
-        <v>348</v>
+        <v>351</v>
       </c>
       <c r="H94" s="1" t="s">
-        <v>397</v>
+        <v>400</v>
       </c>
       <c r="I94">
         <f>F94*VALUE(LEFT(H94, FIND(":", H94)-1))</f>
@@ -5642,7 +5666,7 @@
         <v>1</v>
       </c>
       <c r="H95" s="1" t="s">
-        <v>398</v>
+        <v>401</v>
       </c>
       <c r="I95">
         <f>F95*VALUE(LEFT(H95, FIND(":", H95)-1))</f>
@@ -5671,7 +5695,7 @@
         <v>1</v>
       </c>
       <c r="H96" s="1" t="s">
-        <v>409</v>
+        <v>412</v>
       </c>
       <c r="I96">
         <f>F96*VALUE(LEFT(H96, FIND(":", H96)-1))</f>
@@ -5700,7 +5724,7 @@
         <v>1</v>
       </c>
       <c r="H97" s="1" t="s">
-        <v>398</v>
+        <v>401</v>
       </c>
       <c r="I97">
         <f>F97*VALUE(LEFT(H97, FIND(":", H97)-1))</f>
@@ -5729,7 +5753,7 @@
         <v>1</v>
       </c>
       <c r="H98" s="1" t="s">
-        <v>398</v>
+        <v>401</v>
       </c>
       <c r="I98">
         <f>F98*VALUE(LEFT(H98, FIND(":", H98)-1))</f>
@@ -5762,7 +5786,7 @@
         <v>1</v>
       </c>
       <c r="H99" s="1" t="s">
-        <v>398</v>
+        <v>401</v>
       </c>
       <c r="I99">
         <f>F99*VALUE(LEFT(H99, FIND(":", H99)-1))</f>
@@ -5791,7 +5815,7 @@
         <v>1</v>
       </c>
       <c r="H100" s="1" t="s">
-        <v>398</v>
+        <v>401</v>
       </c>
       <c r="I100">
         <f>F100*VALUE(LEFT(H100, FIND(":", H100)-1))</f>
@@ -5820,7 +5844,7 @@
         <v>1</v>
       </c>
       <c r="H101" s="1" t="s">
-        <v>398</v>
+        <v>401</v>
       </c>
       <c r="I101">
         <f>F101*VALUE(LEFT(H101, FIND(":", H101)-1))</f>
@@ -5849,7 +5873,7 @@
         <v>1</v>
       </c>
       <c r="H102" s="1" t="s">
-        <v>398</v>
+        <v>401</v>
       </c>
       <c r="I102">
         <f>F102*VALUE(LEFT(H102, FIND(":", H102)-1))</f>
@@ -5878,7 +5902,7 @@
         <v>1</v>
       </c>
       <c r="H103" s="1" t="s">
-        <v>410</v>
+        <v>413</v>
       </c>
       <c r="I103">
         <f>F103*VALUE(LEFT(H103, FIND(":", H103)-1))</f>
@@ -5907,7 +5931,7 @@
         <v>1</v>
       </c>
       <c r="H104" s="1" t="s">
-        <v>398</v>
+        <v>401</v>
       </c>
       <c r="I104">
         <f>F104*VALUE(LEFT(H104, FIND(":", H104)-1))</f>
@@ -5938,7 +5962,7 @@
         <v>1</v>
       </c>
       <c r="H105" s="1" t="s">
-        <v>403</v>
+        <v>406</v>
       </c>
       <c r="I105">
         <f>F105*VALUE(LEFT(H105, FIND(":", H105)-1))</f>
@@ -5967,7 +5991,7 @@
         <v>1</v>
       </c>
       <c r="H106" s="1" t="s">
-        <v>403</v>
+        <v>406</v>
       </c>
       <c r="I106">
         <f>F106*VALUE(LEFT(H106, FIND(":", H106)-1))</f>
@@ -5996,7 +6020,7 @@
         <v>1</v>
       </c>
       <c r="H107" s="1" t="s">
-        <v>398</v>
+        <v>401</v>
       </c>
       <c r="I107">
         <f>F107*VALUE(LEFT(H107, FIND(":", H107)-1))</f>
@@ -6025,7 +6049,7 @@
         <v>1</v>
       </c>
       <c r="H108" s="1" t="s">
-        <v>398</v>
+        <v>401</v>
       </c>
       <c r="I108">
         <f>F108*VALUE(LEFT(H108, FIND(":", H108)-1))</f>
@@ -6054,7 +6078,7 @@
         <v>1</v>
       </c>
       <c r="H109" s="1" t="s">
-        <v>398</v>
+        <v>401</v>
       </c>
       <c r="I109">
         <f>F109*VALUE(LEFT(H109, FIND(":", H109)-1))</f>
@@ -6083,7 +6107,7 @@
         <v>1</v>
       </c>
       <c r="H110" s="1" t="s">
-        <v>398</v>
+        <v>401</v>
       </c>
       <c r="I110">
         <f>F110*VALUE(LEFT(H110, FIND(":", H110)-1))</f>
@@ -6114,7 +6138,7 @@
         <v>1</v>
       </c>
       <c r="H111" s="1" t="s">
-        <v>398</v>
+        <v>401</v>
       </c>
       <c r="I111">
         <f>F111*VALUE(LEFT(H111, FIND(":", H111)-1))</f>
@@ -6143,10 +6167,10 @@
         <v>1</v>
       </c>
       <c r="G112" s="1" t="s">
-        <v>349</v>
+        <v>352</v>
       </c>
       <c r="H112" s="1" t="s">
-        <v>397</v>
+        <v>400</v>
       </c>
       <c r="I112">
         <f>F112*VALUE(LEFT(H112, FIND(":", H112)-1))</f>
@@ -6175,7 +6199,7 @@
         <v>1</v>
       </c>
       <c r="H113" s="1" t="s">
-        <v>411</v>
+        <v>414</v>
       </c>
       <c r="I113">
         <f>F113*VALUE(LEFT(H113, FIND(":", H113)-1))</f>
@@ -6204,10 +6228,10 @@
         <v>1</v>
       </c>
       <c r="G114" s="1" t="s">
-        <v>350</v>
+        <v>353</v>
       </c>
       <c r="H114" s="1" t="s">
-        <v>405</v>
+        <v>408</v>
       </c>
       <c r="I114">
         <f>F114*VALUE(LEFT(H114, FIND(":", H114)-1))</f>
@@ -6236,7 +6260,7 @@
         <v>1</v>
       </c>
       <c r="H115" s="1" t="s">
-        <v>412</v>
+        <v>415</v>
       </c>
       <c r="I115">
         <f>F115*VALUE(LEFT(H115, FIND(":", H115)-1))</f>
@@ -6265,10 +6289,10 @@
         <v>1</v>
       </c>
       <c r="G116" s="1" t="s">
-        <v>351</v>
+        <v>354</v>
       </c>
       <c r="H116" s="1" t="s">
-        <v>397</v>
+        <v>400</v>
       </c>
       <c r="I116">
         <f>F116*VALUE(LEFT(H116, FIND(":", H116)-1))</f>
@@ -6299,10 +6323,10 @@
         <v>1</v>
       </c>
       <c r="G117" s="1" t="s">
-        <v>352</v>
+        <v>355</v>
       </c>
       <c r="H117" s="1" t="s">
-        <v>397</v>
+        <v>400</v>
       </c>
       <c r="I117">
         <f>F117*VALUE(LEFT(H117, FIND(":", H117)-1))</f>
@@ -6331,10 +6355,10 @@
         <v>1</v>
       </c>
       <c r="G118" s="1" t="s">
-        <v>353</v>
+        <v>356</v>
       </c>
       <c r="H118" s="1" t="s">
-        <v>397</v>
+        <v>400</v>
       </c>
       <c r="I118">
         <f>F118*VALUE(LEFT(H118, FIND(":", H118)-1))</f>
@@ -6363,10 +6387,10 @@
         <v>1</v>
       </c>
       <c r="G119" s="1" t="s">
-        <v>354</v>
+        <v>357</v>
       </c>
       <c r="H119" s="1" t="s">
-        <v>397</v>
+        <v>400</v>
       </c>
       <c r="I119">
         <f>F119*VALUE(LEFT(H119, FIND(":", H119)-1))</f>
@@ -6395,10 +6419,10 @@
         <v>1</v>
       </c>
       <c r="G120" s="1" t="s">
-        <v>355</v>
+        <v>358</v>
       </c>
       <c r="H120" s="1" t="s">
-        <v>397</v>
+        <v>400</v>
       </c>
       <c r="I120">
         <f>F120*VALUE(LEFT(H120, FIND(":", H120)-1))</f>
@@ -6427,10 +6451,10 @@
         <v>1</v>
       </c>
       <c r="G121" s="1" t="s">
-        <v>356</v>
+        <v>359</v>
       </c>
       <c r="H121" s="1" t="s">
-        <v>397</v>
+        <v>400</v>
       </c>
       <c r="I121">
         <f>F121*VALUE(LEFT(H121, FIND(":", H121)-1))</f>
@@ -6459,7 +6483,7 @@
         <v>1</v>
       </c>
       <c r="H122" s="1" t="s">
-        <v>405</v>
+        <v>408</v>
       </c>
       <c r="I122">
         <f>F122*VALUE(LEFT(H122, FIND(":", H122)-1))</f>
@@ -6488,10 +6512,10 @@
         <v>1</v>
       </c>
       <c r="G123" s="1" t="s">
-        <v>357</v>
+        <v>360</v>
       </c>
       <c r="H123" s="1" t="s">
-        <v>397</v>
+        <v>400</v>
       </c>
       <c r="I123">
         <f>F123*VALUE(LEFT(H123, FIND(":", H123)-1))</f>
@@ -6522,10 +6546,10 @@
         <v>1</v>
       </c>
       <c r="G124" s="1" t="s">
-        <v>358</v>
+        <v>361</v>
       </c>
       <c r="H124" s="1" t="s">
-        <v>397</v>
+        <v>400</v>
       </c>
       <c r="I124">
         <f>F124*VALUE(LEFT(H124, FIND(":", H124)-1))</f>
@@ -6554,10 +6578,10 @@
         <v>1</v>
       </c>
       <c r="G125" s="1" t="s">
-        <v>359</v>
+        <v>362</v>
       </c>
       <c r="H125" s="1" t="s">
-        <v>397</v>
+        <v>400</v>
       </c>
       <c r="I125">
         <f>F125*VALUE(LEFT(H125, FIND(":", H125)-1))</f>
@@ -6586,10 +6610,10 @@
         <v>1</v>
       </c>
       <c r="G126" s="1" t="s">
-        <v>360</v>
+        <v>363</v>
       </c>
       <c r="H126" s="1" t="s">
-        <v>397</v>
+        <v>400</v>
       </c>
       <c r="I126">
         <f>F126*VALUE(LEFT(H126, FIND(":", H126)-1))</f>
@@ -6618,10 +6642,10 @@
         <v>1</v>
       </c>
       <c r="G127" s="1" t="s">
-        <v>361</v>
+        <v>364</v>
       </c>
       <c r="H127" s="1" t="s">
-        <v>397</v>
+        <v>400</v>
       </c>
       <c r="I127">
         <f>F127*VALUE(LEFT(H127, FIND(":", H127)-1))</f>
@@ -6650,10 +6674,10 @@
         <v>1</v>
       </c>
       <c r="G128" s="1" t="s">
-        <v>362</v>
+        <v>365</v>
       </c>
       <c r="H128" s="1" t="s">
-        <v>397</v>
+        <v>400</v>
       </c>
       <c r="I128">
         <f>F128*VALUE(LEFT(H128, FIND(":", H128)-1))</f>
@@ -6682,7 +6706,7 @@
         <v>1</v>
       </c>
       <c r="H129" s="1" t="s">
-        <v>411</v>
+        <v>414</v>
       </c>
       <c r="I129">
         <f>F129*VALUE(LEFT(H129, FIND(":", H129)-1))</f>
@@ -6715,7 +6739,7 @@
         <v>1</v>
       </c>
       <c r="H130" s="1" t="s">
-        <v>398</v>
+        <v>401</v>
       </c>
       <c r="I130">
         <f>F130*VALUE(LEFT(H130, FIND(":", H130)-1))</f>
@@ -6744,7 +6768,7 @@
         <v>1</v>
       </c>
       <c r="H131" s="1" t="s">
-        <v>398</v>
+        <v>401</v>
       </c>
       <c r="I131">
         <f>F131*VALUE(LEFT(H131, FIND(":", H131)-1))</f>
@@ -6773,7 +6797,7 @@
         <v>1</v>
       </c>
       <c r="H132" s="1" t="s">
-        <v>398</v>
+        <v>401</v>
       </c>
       <c r="I132">
         <f>F132*VALUE(LEFT(H132, FIND(":", H132)-1))</f>
@@ -6802,7 +6826,7 @@
         <v>1</v>
       </c>
       <c r="H133" s="1" t="s">
-        <v>413</v>
+        <v>416</v>
       </c>
       <c r="I133">
         <f>F133*VALUE(LEFT(H133, FIND(":", H133)-1))</f>
@@ -6831,7 +6855,7 @@
         <v>1</v>
       </c>
       <c r="H134" s="1" t="s">
-        <v>398</v>
+        <v>401</v>
       </c>
       <c r="I134">
         <f>F134*VALUE(LEFT(H134, FIND(":", H134)-1))</f>
@@ -6994,10 +7018,10 @@
       <formula1>"0: No documented method,10: Documented method of assessing modernization efforts"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H42">
-      <formula1>"0: Not done,10: Completed"</formula1>
+      <formula1>"0: No items completed,2: 1 item completed,4: 2 items completed,6: 3 items completed,8: 4 items completed,10: 5 items completed"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H43">
-      <formula1>"0: Not done,10: Completed"</formula1>
+      <formula1>"0: No items completed,3: 1 item completed,5: 2 items completed,8: 3 items completed,10: 4 items completed"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H44">
       <formula1>"0: Not done,10: Completed"</formula1>

</xml_diff>